<commit_message>
Added new field data. New code that takes 2 mins from 3 min enclosures. Graphs from unannotated data also plotted to check for congruency
</commit_message>
<xml_diff>
--- a/Field_Data/Field_Data.xlsx
+++ b/Field_Data/Field_Data.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11268"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11265"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -423,17 +423,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J136"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="8" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="8" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.5703125" customWidth="1"/>
+    <col min="10" max="10" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -465,247 +466,799 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="2">
         <v>45810</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C2" s="3">
+        <v>0.40138888888888885</v>
+      </c>
+      <c r="D2">
+        <v>30</v>
+      </c>
+      <c r="E2">
+        <v>-6</v>
+      </c>
+      <c r="F2">
+        <v>-6</v>
+      </c>
+      <c r="G2">
+        <v>-6</v>
+      </c>
+      <c r="H2">
+        <v>-6.5</v>
+      </c>
+      <c r="I2">
+        <v>0.5</v>
+      </c>
+      <c r="J2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="2">
         <v>45810</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C3" s="3">
+        <v>0.40833333333333338</v>
+      </c>
+      <c r="D3">
+        <v>30</v>
+      </c>
+      <c r="E3">
+        <v>-6</v>
+      </c>
+      <c r="I3">
+        <v>0.5</v>
+      </c>
+      <c r="J3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="2">
         <v>45810</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C4" s="3">
+        <v>0.41180555555555554</v>
+      </c>
+      <c r="D4">
+        <v>30</v>
+      </c>
+      <c r="E4">
+        <v>-6</v>
+      </c>
+      <c r="I4">
+        <v>0.5</v>
+      </c>
+      <c r="J4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="2">
         <v>45810</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C5" s="3">
+        <v>0.4145833333333333</v>
+      </c>
+      <c r="D5">
+        <v>30</v>
+      </c>
+      <c r="E5">
+        <v>-6</v>
+      </c>
+      <c r="I5">
+        <v>0.5</v>
+      </c>
+      <c r="J5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
       <c r="B6" s="2">
         <v>45810</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C6" s="3">
+        <v>0.41736111111111113</v>
+      </c>
+      <c r="D6">
+        <v>30</v>
+      </c>
+      <c r="E6">
+        <v>-5.5</v>
+      </c>
+      <c r="F6">
+        <v>-6</v>
+      </c>
+      <c r="G6">
+        <v>-6</v>
+      </c>
+      <c r="H6">
+        <v>-5.8</v>
+      </c>
+      <c r="I6">
+        <v>0.5</v>
+      </c>
+      <c r="J6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
       <c r="B7" s="2">
         <v>45810</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C7" s="3">
+        <v>0.42083333333333334</v>
+      </c>
+      <c r="D7">
+        <v>30</v>
+      </c>
+      <c r="E7">
+        <v>-6</v>
+      </c>
+      <c r="I7">
+        <v>0.5</v>
+      </c>
+      <c r="J7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="2">
         <v>45810</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C8" s="3">
+        <v>0.4236111111111111</v>
+      </c>
+      <c r="D8">
+        <v>30</v>
+      </c>
+      <c r="E8">
+        <v>-6</v>
+      </c>
+      <c r="I8">
+        <v>0.5</v>
+      </c>
+      <c r="J8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>14</v>
       </c>
       <c r="B9" s="2">
         <v>45810</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C9" s="3">
+        <v>0.42777777777777781</v>
+      </c>
+      <c r="D9">
+        <v>30</v>
+      </c>
+      <c r="E9">
+        <v>-6</v>
+      </c>
+      <c r="F9">
+        <v>-6.5</v>
+      </c>
+      <c r="G9">
+        <v>-6.3</v>
+      </c>
+      <c r="H9">
+        <v>-6.5</v>
+      </c>
+      <c r="I9">
+        <v>0.5</v>
+      </c>
+      <c r="J9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>15</v>
       </c>
       <c r="B10" s="2">
         <v>45810</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C10" s="3">
+        <v>0.43055555555555558</v>
+      </c>
+      <c r="D10">
+        <v>30</v>
+      </c>
+      <c r="E10">
+        <v>-6.5</v>
+      </c>
+      <c r="F10">
+        <v>-6.5</v>
+      </c>
+      <c r="G10">
+        <v>-6.5</v>
+      </c>
+      <c r="H10">
+        <v>-6.8</v>
+      </c>
+      <c r="I10">
+        <v>0.5</v>
+      </c>
+      <c r="J10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>16</v>
       </c>
       <c r="B11" s="2">
         <v>45810</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C11" s="3">
+        <v>0.43333333333333302</v>
+      </c>
+      <c r="D11">
+        <v>30</v>
+      </c>
+      <c r="E11">
+        <v>-6</v>
+      </c>
+      <c r="I11">
+        <v>0.5</v>
+      </c>
+      <c r="J11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>17</v>
       </c>
       <c r="B12" s="2">
         <v>45810</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C12" s="3">
+        <v>0.43645833333333334</v>
+      </c>
+      <c r="D12">
+        <v>30</v>
+      </c>
+      <c r="E12">
+        <v>-6.5</v>
+      </c>
+      <c r="F12">
+        <v>-6.5</v>
+      </c>
+      <c r="G12">
+        <v>-6</v>
+      </c>
+      <c r="H12">
+        <v>-6.3</v>
+      </c>
+      <c r="I12">
+        <v>0.5</v>
+      </c>
+      <c r="J12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>18</v>
       </c>
       <c r="B13" s="2">
         <v>45810</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C13" s="3">
+        <v>0.43958333333333338</v>
+      </c>
+      <c r="D13">
+        <v>30</v>
+      </c>
+      <c r="E13">
+        <v>-7</v>
+      </c>
+      <c r="F13">
+        <v>-7</v>
+      </c>
+      <c r="G13">
+        <v>-7</v>
+      </c>
+      <c r="H13">
+        <v>-6.5</v>
+      </c>
+      <c r="I13">
+        <v>0.5</v>
+      </c>
+      <c r="J13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>19</v>
       </c>
       <c r="B14" s="2">
         <v>45810</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C14" s="3">
+        <v>0.44444444444444442</v>
+      </c>
+      <c r="D14">
+        <v>30</v>
+      </c>
+      <c r="E14">
+        <v>-6.9</v>
+      </c>
+      <c r="F14">
+        <v>-6.9</v>
+      </c>
+      <c r="I14">
+        <v>0.5</v>
+      </c>
+      <c r="J14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>20</v>
       </c>
       <c r="B15" s="2">
         <v>45810</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C15" s="3">
+        <v>0.44791666666666669</v>
+      </c>
+      <c r="D15">
+        <v>30</v>
+      </c>
+      <c r="E15">
+        <v>-7</v>
+      </c>
+      <c r="F15">
+        <v>-7</v>
+      </c>
+      <c r="G15">
+        <v>-7.3</v>
+      </c>
+      <c r="H15">
+        <v>-7.5</v>
+      </c>
+      <c r="I15">
+        <v>0.5</v>
+      </c>
+      <c r="J15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>21</v>
       </c>
       <c r="B16" s="2">
         <v>45810</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C16" s="3">
+        <v>0.4513888888888889</v>
+      </c>
+      <c r="D16">
+        <v>30</v>
+      </c>
+      <c r="E16">
+        <v>-7</v>
+      </c>
+      <c r="F16">
+        <v>-7</v>
+      </c>
+      <c r="G16">
+        <v>-7.5</v>
+      </c>
+      <c r="H16">
+        <v>-7</v>
+      </c>
+      <c r="I16">
+        <v>0.5</v>
+      </c>
+      <c r="J16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="2">
         <v>45817</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C17" s="3">
+        <v>0.38819444444444445</v>
+      </c>
+      <c r="D17">
+        <v>31</v>
+      </c>
+      <c r="E17">
+        <v>-5.6</v>
+      </c>
+      <c r="I17">
+        <v>0.5</v>
+      </c>
+      <c r="J17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>8</v>
       </c>
       <c r="B18" s="2">
         <v>45817</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C18" s="3">
+        <v>0.39444444444444443</v>
+      </c>
+      <c r="D18">
+        <v>31</v>
+      </c>
+      <c r="E18">
+        <v>-5.3</v>
+      </c>
+      <c r="I18">
+        <v>0.5</v>
+      </c>
+      <c r="J18">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>9</v>
       </c>
       <c r="B19" s="2">
         <v>45817</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C19" s="3">
+        <v>0.39861111111111108</v>
+      </c>
+      <c r="D19">
+        <v>31</v>
+      </c>
+      <c r="E19">
+        <v>-5.2</v>
+      </c>
+      <c r="I19">
+        <v>0.5</v>
+      </c>
+      <c r="J19">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>10</v>
       </c>
       <c r="B20" s="2">
         <v>45817</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C20" s="3">
+        <v>0.40277777777777801</v>
+      </c>
+      <c r="D20">
+        <v>31</v>
+      </c>
+      <c r="E20">
+        <v>-5.0999999999999996</v>
+      </c>
+      <c r="I20">
+        <v>0.5</v>
+      </c>
+      <c r="J20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>11</v>
       </c>
       <c r="B21" s="2">
         <v>45817</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C21" s="3">
+        <v>0.406944444444444</v>
+      </c>
+      <c r="D21">
+        <v>31</v>
+      </c>
+      <c r="E21">
+        <v>-5.3</v>
+      </c>
+      <c r="I21">
+        <v>0.5</v>
+      </c>
+      <c r="J21">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>12</v>
       </c>
       <c r="B22" s="2">
         <v>45817</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C22" s="3">
+        <v>0.41250000000000003</v>
+      </c>
+      <c r="D22">
+        <v>31</v>
+      </c>
+      <c r="E22">
+        <v>-5.3</v>
+      </c>
+      <c r="F22">
+        <v>-5.7</v>
+      </c>
+      <c r="G22">
+        <v>-5.4</v>
+      </c>
+      <c r="H22">
+        <v>-5.7</v>
+      </c>
+      <c r="I22">
+        <v>0.5</v>
+      </c>
+      <c r="J22">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>13</v>
       </c>
       <c r="B23" s="2">
         <v>45817</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C23" s="3">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="D23">
+        <v>31</v>
+      </c>
+      <c r="E23">
+        <v>-5.8</v>
+      </c>
+      <c r="I23">
+        <v>0.5</v>
+      </c>
+      <c r="J23">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>14</v>
       </c>
       <c r="B24" s="2">
         <v>45817</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C24" s="3">
+        <v>0.420833333333333</v>
+      </c>
+      <c r="D24">
+        <v>31</v>
+      </c>
+      <c r="E24">
+        <v>-5.8</v>
+      </c>
+      <c r="F24">
+        <v>-5.4</v>
+      </c>
+      <c r="G24">
+        <v>-5.5</v>
+      </c>
+      <c r="H24">
+        <v>-5.7</v>
+      </c>
+      <c r="I24">
+        <v>0.5</v>
+      </c>
+      <c r="J24">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>15</v>
       </c>
       <c r="B25" s="2">
         <v>45817</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C25" s="3">
+        <v>0.42499999999999999</v>
+      </c>
+      <c r="D25">
+        <v>31</v>
+      </c>
+      <c r="E25">
+        <v>-5.8</v>
+      </c>
+      <c r="I25">
+        <v>0.5</v>
+      </c>
+      <c r="J25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>16</v>
       </c>
       <c r="B26" s="2">
         <v>45817</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C26" s="3">
+        <v>0.42916666666666697</v>
+      </c>
+      <c r="D26">
+        <v>31</v>
+      </c>
+      <c r="E26">
+        <v>-5.4</v>
+      </c>
+      <c r="F26">
+        <v>-5</v>
+      </c>
+      <c r="G26">
+        <v>-5.3</v>
+      </c>
+      <c r="H26">
+        <v>-5.4</v>
+      </c>
+      <c r="I26">
+        <v>0.5</v>
+      </c>
+      <c r="J26">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>17</v>
       </c>
       <c r="B27" s="2">
         <v>45817</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C27" s="3">
+        <v>0.43402777777777773</v>
+      </c>
+      <c r="D27">
+        <v>31</v>
+      </c>
+      <c r="E27">
+        <v>-4.7</v>
+      </c>
+      <c r="I27">
+        <v>0.5</v>
+      </c>
+      <c r="J27">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>18</v>
       </c>
       <c r="B28" s="2">
         <v>45817</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C28" s="3">
+        <v>0.4381944444444445</v>
+      </c>
+      <c r="D28">
+        <v>31</v>
+      </c>
+      <c r="E28">
+        <v>-5.9</v>
+      </c>
+      <c r="I28">
+        <v>0.5</v>
+      </c>
+      <c r="J28">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>19</v>
       </c>
       <c r="B29" s="2">
         <v>45817</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C29" s="3">
+        <v>0.44236111111111098</v>
+      </c>
+      <c r="D29">
+        <v>31</v>
+      </c>
+      <c r="E29">
+        <v>-6.6</v>
+      </c>
+      <c r="I29">
+        <v>0.5</v>
+      </c>
+      <c r="J29">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>20</v>
       </c>
       <c r="B30" s="2">
         <v>45817</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C30" s="3">
+        <v>0.44722222222222219</v>
+      </c>
+      <c r="D30">
+        <v>31</v>
+      </c>
+      <c r="E30">
+        <v>-6.1</v>
+      </c>
+      <c r="I30">
+        <v>0.5</v>
+      </c>
+      <c r="J30">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>21</v>
       </c>
       <c r="B31" s="2">
         <v>45817</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C31" s="3">
+        <v>0.4513888888888889</v>
+      </c>
+      <c r="D31">
+        <v>31</v>
+      </c>
+      <c r="E31">
+        <v>-5.8</v>
+      </c>
+      <c r="I31">
+        <v>0.5</v>
+      </c>
+      <c r="J31">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>7</v>
       </c>
@@ -728,7 +1281,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>8</v>
       </c>
@@ -751,7 +1304,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>9</v>
       </c>
@@ -774,7 +1327,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>10</v>
       </c>
@@ -797,7 +1350,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>11</v>
       </c>
@@ -820,7 +1373,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>12</v>
       </c>
@@ -846,7 +1399,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>13</v>
       </c>
@@ -878,7 +1431,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>14</v>
       </c>
@@ -901,7 +1454,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>15</v>
       </c>
@@ -933,7 +1486,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>16</v>
       </c>
@@ -956,7 +1509,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>17</v>
       </c>
@@ -979,7 +1532,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>18</v>
       </c>
@@ -1002,7 +1555,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>19</v>
       </c>
@@ -1025,7 +1578,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>20</v>
       </c>
@@ -1048,7 +1601,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>21</v>
       </c>
@@ -1071,7 +1624,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>7</v>
       </c>
@@ -1094,7 +1647,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>8</v>
       </c>
@@ -1117,7 +1670,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>9</v>
       </c>
@@ -1140,7 +1693,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>10</v>
       </c>
@@ -1163,7 +1716,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>11</v>
       </c>
@@ -1195,7 +1748,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>12</v>
       </c>
@@ -1227,7 +1780,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>13</v>
       </c>
@@ -1250,7 +1803,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>14</v>
       </c>
@@ -1282,7 +1835,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>15</v>
       </c>
@@ -1305,7 +1858,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>16</v>
       </c>
@@ -1337,7 +1890,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>17</v>
       </c>
@@ -1360,7 +1913,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>18</v>
       </c>
@@ -1383,7 +1936,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>19</v>
       </c>
@@ -1406,7 +1959,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>20</v>
       </c>
@@ -1438,7 +1991,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>21</v>
       </c>
@@ -1461,7 +2014,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>7</v>
       </c>
@@ -1493,7 +2046,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>8</v>
       </c>
@@ -1519,7 +2072,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>9</v>
       </c>
@@ -1551,7 +2104,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>10</v>
       </c>
@@ -1583,7 +2136,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>11</v>
       </c>
@@ -1606,7 +2159,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>12</v>
       </c>
@@ -1629,7 +2182,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>13</v>
       </c>
@@ -1652,7 +2205,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>14</v>
       </c>
@@ -1675,7 +2228,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>15</v>
       </c>
@@ -1698,7 +2251,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>16</v>
       </c>
@@ -1721,7 +2274,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>17</v>
       </c>
@@ -1744,7 +2297,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>18</v>
       </c>
@@ -1776,7 +2329,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>19</v>
       </c>
@@ -1799,7 +2352,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>20</v>
       </c>
@@ -1825,7 +2378,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>21</v>
       </c>
@@ -1848,7 +2401,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>7</v>
       </c>
@@ -1871,7 +2424,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -1894,7 +2447,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>9</v>
       </c>
@@ -1926,7 +2479,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>10</v>
       </c>
@@ -1958,7 +2511,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>11</v>
       </c>
@@ -1990,7 +2543,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>12</v>
       </c>
@@ -2013,7 +2566,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>13</v>
       </c>
@@ -2036,7 +2589,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>14</v>
       </c>
@@ -2068,7 +2621,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>15</v>
       </c>
@@ -2076,7 +2629,7 @@
         <v>45849</v>
       </c>
       <c r="C85" s="1">
-        <v>0.42291666666666666</v>
+        <v>0.42499999999999999</v>
       </c>
       <c r="D85">
         <v>28.9</v>
@@ -2091,7 +2644,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>16</v>
       </c>
@@ -2123,7 +2676,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>17</v>
       </c>
@@ -2155,7 +2708,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>18</v>
       </c>
@@ -2187,7 +2740,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>19</v>
       </c>
@@ -2219,7 +2772,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>20</v>
       </c>
@@ -2242,7 +2795,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>21</v>
       </c>
@@ -2265,364 +2818,1198 @@
         <v>4</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>7</v>
       </c>
       <c r="B92" s="2">
         <v>45856</v>
       </c>
-    </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C92" s="3">
+        <v>0.3923611111111111</v>
+      </c>
+      <c r="D92">
+        <v>24.1</v>
+      </c>
+      <c r="E92">
+        <v>-7</v>
+      </c>
+      <c r="I92">
+        <v>2</v>
+      </c>
+      <c r="J92">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>8</v>
       </c>
       <c r="B93" s="2">
         <v>45856</v>
       </c>
-    </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C93" s="3">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="D93">
+        <v>23.4</v>
+      </c>
+      <c r="E93">
+        <v>-7.2</v>
+      </c>
+      <c r="I93">
+        <v>2</v>
+      </c>
+      <c r="J93">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>9</v>
       </c>
       <c r="B94" s="2">
         <v>45856</v>
       </c>
-    </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C94" s="3">
+        <v>0.39930555555555602</v>
+      </c>
+      <c r="D94">
+        <v>23.9</v>
+      </c>
+      <c r="E94">
+        <v>-7</v>
+      </c>
+      <c r="I94">
+        <v>2</v>
+      </c>
+      <c r="J94">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>10</v>
       </c>
       <c r="B95" s="2">
         <v>45856</v>
       </c>
-    </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C95" s="3">
+        <v>0.40277777777777801</v>
+      </c>
+      <c r="D95">
+        <v>23.8</v>
+      </c>
+      <c r="E95">
+        <v>-7</v>
+      </c>
+      <c r="I95">
+        <v>2</v>
+      </c>
+      <c r="J95">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>11</v>
       </c>
       <c r="B96" s="2">
         <v>45856</v>
       </c>
-    </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C96" s="3">
+        <v>0.40625</v>
+      </c>
+      <c r="D96">
+        <v>25.5</v>
+      </c>
+      <c r="E96">
+        <v>-7</v>
+      </c>
+      <c r="I96">
+        <v>2</v>
+      </c>
+      <c r="J96">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>12</v>
       </c>
       <c r="B97" s="2">
         <v>45856</v>
       </c>
-    </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C97" s="3">
+        <v>0.40972222222222199</v>
+      </c>
+      <c r="D97">
+        <v>24.4</v>
+      </c>
+      <c r="E97">
+        <v>-8.5</v>
+      </c>
+      <c r="F97">
+        <v>-7.7</v>
+      </c>
+      <c r="G97">
+        <v>-7.7</v>
+      </c>
+      <c r="H97">
+        <v>-9</v>
+      </c>
+      <c r="I97">
+        <v>2</v>
+      </c>
+      <c r="J97">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>13</v>
       </c>
       <c r="B98" s="2">
         <v>45856</v>
       </c>
-    </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C98" s="3">
+        <v>0.41319444444444398</v>
+      </c>
+      <c r="D98">
+        <v>24.3</v>
+      </c>
+      <c r="E98">
+        <v>-7</v>
+      </c>
+      <c r="F98">
+        <v>-7.5</v>
+      </c>
+      <c r="G98">
+        <v>-7.3</v>
+      </c>
+      <c r="H98">
+        <v>-7</v>
+      </c>
+      <c r="I98">
+        <v>2</v>
+      </c>
+      <c r="J98">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>14</v>
       </c>
       <c r="B99" s="2">
         <v>45856</v>
       </c>
-    </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C99" s="3">
+        <v>0.41666666666666702</v>
+      </c>
+      <c r="D99">
+        <v>24.5</v>
+      </c>
+      <c r="E99">
+        <v>-7.5</v>
+      </c>
+      <c r="F99">
+        <v>-7.5</v>
+      </c>
+      <c r="I99">
+        <v>2</v>
+      </c>
+      <c r="J99">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>15</v>
       </c>
       <c r="B100" s="2">
         <v>45856</v>
       </c>
-    </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C100" s="3">
+        <v>0.42013888888888901</v>
+      </c>
+      <c r="D100">
+        <v>24.2</v>
+      </c>
+      <c r="E100">
+        <v>-7.8</v>
+      </c>
+      <c r="I100">
+        <v>2</v>
+      </c>
+      <c r="J100">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>16</v>
       </c>
       <c r="B101" s="2">
         <v>45856</v>
       </c>
-    </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C101" s="3">
+        <v>0.42361111111111099</v>
+      </c>
+      <c r="D101">
+        <v>24.4</v>
+      </c>
+      <c r="E101">
+        <v>-7.2</v>
+      </c>
+      <c r="I101">
+        <v>2</v>
+      </c>
+      <c r="J101">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>17</v>
       </c>
       <c r="B102" s="2">
         <v>45856</v>
       </c>
-    </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C102" s="3">
+        <v>0.42708333333333298</v>
+      </c>
+      <c r="D102">
+        <v>25.1</v>
+      </c>
+      <c r="E102">
+        <v>-7.5</v>
+      </c>
+      <c r="F102">
+        <v>-8</v>
+      </c>
+      <c r="G102">
+        <v>-7</v>
+      </c>
+      <c r="H102">
+        <v>-8</v>
+      </c>
+      <c r="I102">
+        <v>2</v>
+      </c>
+      <c r="J102">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>18</v>
       </c>
       <c r="B103" s="2">
         <v>45856</v>
       </c>
-    </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C103" s="3">
+        <v>0.43055555555555503</v>
+      </c>
+      <c r="D103">
+        <v>24.9</v>
+      </c>
+      <c r="E103">
+        <v>-8</v>
+      </c>
+      <c r="I103">
+        <v>2</v>
+      </c>
+      <c r="J103">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>19</v>
       </c>
       <c r="B104" s="2">
         <v>45856</v>
       </c>
-    </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C104" s="3">
+        <v>0.43402777777777801</v>
+      </c>
+      <c r="D104">
+        <v>24.6</v>
+      </c>
+      <c r="E104">
+        <v>-8</v>
+      </c>
+      <c r="I104">
+        <v>2</v>
+      </c>
+      <c r="J104">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>20</v>
       </c>
       <c r="B105" s="2">
         <v>45856</v>
       </c>
-    </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C105" s="3">
+        <v>0.4375</v>
+      </c>
+      <c r="D105">
+        <v>25.4</v>
+      </c>
+      <c r="E105">
+        <v>-8</v>
+      </c>
+      <c r="I105">
+        <v>2</v>
+      </c>
+      <c r="J105">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>21</v>
       </c>
       <c r="B106" s="2">
         <v>45856</v>
       </c>
-    </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C106" s="3">
+        <v>0.44305555555555554</v>
+      </c>
+      <c r="D106">
+        <v>24.8</v>
+      </c>
+      <c r="E106">
+        <v>-7.5</v>
+      </c>
+      <c r="F106">
+        <v>-8</v>
+      </c>
+      <c r="G106">
+        <v>-8.5</v>
+      </c>
+      <c r="H106">
+        <v>-8.5</v>
+      </c>
+      <c r="I106">
+        <v>2</v>
+      </c>
+      <c r="J106">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>7</v>
       </c>
       <c r="B107" s="2">
         <v>45863</v>
       </c>
-    </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C107" s="3">
+        <v>0.39999999999999997</v>
+      </c>
+      <c r="D107">
+        <v>22.9</v>
+      </c>
+      <c r="E107">
+        <v>-7</v>
+      </c>
+      <c r="F107">
+        <v>-6.8</v>
+      </c>
+      <c r="G107">
+        <v>-7</v>
+      </c>
+      <c r="H107">
+        <v>-6.8</v>
+      </c>
+      <c r="I107">
+        <v>2</v>
+      </c>
+      <c r="J107">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>8</v>
       </c>
       <c r="B108" s="2">
         <v>45863</v>
       </c>
-    </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C108" s="3">
+        <v>0.40347222222222223</v>
+      </c>
+      <c r="D108">
+        <v>22.1</v>
+      </c>
+      <c r="E108">
+        <v>-6.5</v>
+      </c>
+      <c r="I108">
+        <v>2</v>
+      </c>
+      <c r="J108">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>9</v>
       </c>
       <c r="B109" s="2">
         <v>45863</v>
       </c>
-    </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C109" s="3">
+        <v>0.406944444444444</v>
+      </c>
+      <c r="D109">
+        <v>23.1</v>
+      </c>
+      <c r="E109">
+        <v>-6.5</v>
+      </c>
+      <c r="I109">
+        <v>2</v>
+      </c>
+      <c r="J109">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>10</v>
       </c>
       <c r="B110" s="2">
         <v>45863</v>
       </c>
-    </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C110" s="3">
+        <v>0.41111111111111115</v>
+      </c>
+      <c r="D110">
+        <v>22.2</v>
+      </c>
+      <c r="E110">
+        <v>-7</v>
+      </c>
+      <c r="I110">
+        <v>2</v>
+      </c>
+      <c r="J110">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>11</v>
       </c>
       <c r="B111" s="2">
         <v>45863</v>
       </c>
-    </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C111" s="3">
+        <v>0.4145833333333333</v>
+      </c>
+      <c r="D111">
+        <v>22.5</v>
+      </c>
+      <c r="E111">
+        <v>-7.1</v>
+      </c>
+      <c r="F111">
+        <v>-7.5</v>
+      </c>
+      <c r="G111">
+        <v>-7.4</v>
+      </c>
+      <c r="H111">
+        <v>-7.2</v>
+      </c>
+      <c r="I111">
+        <v>2</v>
+      </c>
+      <c r="J111">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>12</v>
       </c>
       <c r="B112" s="2">
         <v>45863</v>
       </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C112" s="3">
+        <v>0.41805555555555557</v>
+      </c>
+      <c r="D112">
+        <v>23.9</v>
+      </c>
+      <c r="E112">
+        <v>-7.3</v>
+      </c>
+      <c r="I112">
+        <v>2</v>
+      </c>
+      <c r="J112">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>13</v>
       </c>
       <c r="B113" s="2">
         <v>45863</v>
       </c>
-    </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C113" s="3">
+        <v>0.42152777777777778</v>
+      </c>
+      <c r="D113">
+        <v>23.8</v>
+      </c>
+      <c r="E113">
+        <v>-7.3</v>
+      </c>
+      <c r="F113">
+        <v>-7.2</v>
+      </c>
+      <c r="G113">
+        <v>-7.1</v>
+      </c>
+      <c r="H113">
+        <v>-7.3</v>
+      </c>
+      <c r="I113">
+        <v>2</v>
+      </c>
+      <c r="J113">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>14</v>
       </c>
       <c r="B114" s="2">
         <v>45863</v>
       </c>
-    </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C114" s="3">
+        <v>0.42499999999999999</v>
+      </c>
+      <c r="D114">
+        <v>23.9</v>
+      </c>
+      <c r="E114">
+        <v>-6.8</v>
+      </c>
+      <c r="F114">
+        <v>-6.8</v>
+      </c>
+      <c r="I114">
+        <v>2</v>
+      </c>
+      <c r="J114">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>15</v>
       </c>
       <c r="B115" s="2">
         <v>45863</v>
       </c>
-    </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C115" s="3">
+        <v>0.4291666666666667</v>
+      </c>
+      <c r="D115">
+        <v>23.8</v>
+      </c>
+      <c r="E115">
+        <v>-7.2</v>
+      </c>
+      <c r="I115">
+        <v>2</v>
+      </c>
+      <c r="J115">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>16</v>
       </c>
       <c r="B116" s="2">
         <v>45863</v>
       </c>
-    </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C116" s="3">
+        <v>0.43263888888888885</v>
+      </c>
+      <c r="D116">
+        <v>23.9</v>
+      </c>
+      <c r="E116">
+        <v>-6.5</v>
+      </c>
+      <c r="I116">
+        <v>2</v>
+      </c>
+      <c r="J116">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>17</v>
       </c>
       <c r="B117" s="2">
         <v>45863</v>
       </c>
-    </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C117" s="3">
+        <v>0.44097222222222227</v>
+      </c>
+      <c r="D117">
+        <v>24</v>
+      </c>
+      <c r="E117">
+        <v>-6.2</v>
+      </c>
+      <c r="I117">
+        <v>2</v>
+      </c>
+      <c r="J117">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>18</v>
       </c>
       <c r="B118" s="2">
         <v>45863</v>
       </c>
-    </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C118" s="3">
+        <v>0.4458333333333333</v>
+      </c>
+      <c r="D118">
+        <v>23.8</v>
+      </c>
+      <c r="E118">
+        <v>-7.2</v>
+      </c>
+      <c r="I118">
+        <v>2</v>
+      </c>
+      <c r="J118">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>19</v>
       </c>
       <c r="B119" s="2">
         <v>45863</v>
       </c>
-    </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C119" s="3">
+        <v>0.45</v>
+      </c>
+      <c r="D119">
+        <v>22.8</v>
+      </c>
+      <c r="E119">
+        <v>-8</v>
+      </c>
+      <c r="F119">
+        <v>-8.3000000000000007</v>
+      </c>
+      <c r="G119">
+        <v>-8</v>
+      </c>
+      <c r="H119">
+        <v>-8</v>
+      </c>
+      <c r="I119">
+        <v>2</v>
+      </c>
+      <c r="J119">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>20</v>
       </c>
       <c r="B120" s="2">
         <v>45863</v>
       </c>
-    </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C120" s="3">
+        <v>0.45416666666666666</v>
+      </c>
+      <c r="D120">
+        <v>23.2</v>
+      </c>
+      <c r="E120">
+        <v>-7.5</v>
+      </c>
+      <c r="F120">
+        <v>-7.5</v>
+      </c>
+      <c r="I120">
+        <v>2</v>
+      </c>
+      <c r="J120">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>21</v>
       </c>
       <c r="B121" s="2">
         <v>45863</v>
       </c>
-    </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C121" s="3">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D121">
+        <v>23.7</v>
+      </c>
+      <c r="E121">
+        <v>-7.2</v>
+      </c>
+      <c r="I121">
+        <v>2</v>
+      </c>
+      <c r="J121">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>7</v>
       </c>
       <c r="B122" s="2">
         <v>45873</v>
       </c>
-    </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C122" s="3">
+        <v>0.41736111111111113</v>
+      </c>
+      <c r="D122">
+        <v>23.4</v>
+      </c>
+      <c r="E122">
+        <v>-7</v>
+      </c>
+      <c r="F122">
+        <v>-6.5</v>
+      </c>
+      <c r="I122">
+        <v>2</v>
+      </c>
+      <c r="J122">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>8</v>
       </c>
       <c r="B123" s="2">
         <v>45873</v>
       </c>
-    </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C123" s="3">
+        <v>0.42083333333333334</v>
+      </c>
+      <c r="D123">
+        <v>24.1</v>
+      </c>
+      <c r="E123">
+        <v>-6.8</v>
+      </c>
+      <c r="F123">
+        <v>-6.8</v>
+      </c>
+      <c r="G123">
+        <v>-6.6</v>
+      </c>
+      <c r="H123">
+        <v>-6.8</v>
+      </c>
+      <c r="I123">
+        <v>2</v>
+      </c>
+      <c r="J123">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>9</v>
       </c>
       <c r="B124" s="2">
         <v>45873</v>
       </c>
-    </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C124" s="3">
+        <v>0.42430555555555599</v>
+      </c>
+      <c r="D124">
+        <v>23.7</v>
+      </c>
+      <c r="E124">
+        <v>-6.5</v>
+      </c>
+      <c r="I124">
+        <v>2</v>
+      </c>
+      <c r="J124">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>10</v>
       </c>
       <c r="B125" s="2">
         <v>45873</v>
       </c>
-    </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C125" s="3">
+        <v>0.42777777777777798</v>
+      </c>
+      <c r="D125">
+        <v>24.3</v>
+      </c>
+      <c r="E125">
+        <v>-6.5</v>
+      </c>
+      <c r="F125">
+        <v>-6.6</v>
+      </c>
+      <c r="G125">
+        <v>-6.7</v>
+      </c>
+      <c r="H125">
+        <v>-6.8</v>
+      </c>
+      <c r="I125">
+        <v>2</v>
+      </c>
+      <c r="J125">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>11</v>
       </c>
       <c r="B126" s="2">
         <v>45873</v>
       </c>
-    </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C126" s="3">
+        <v>0.43125000000000002</v>
+      </c>
+      <c r="D126">
+        <v>24.3</v>
+      </c>
+      <c r="E126">
+        <v>-6.2</v>
+      </c>
+      <c r="F126">
+        <v>-6.4</v>
+      </c>
+      <c r="G126">
+        <v>-6.2</v>
+      </c>
+      <c r="H126">
+        <v>-7</v>
+      </c>
+      <c r="I126">
+        <v>2</v>
+      </c>
+      <c r="J126">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>12</v>
       </c>
       <c r="B127" s="2">
         <v>45873</v>
       </c>
-    </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C127" s="3">
+        <v>0.43472222222222201</v>
+      </c>
+      <c r="D127">
+        <v>24</v>
+      </c>
+      <c r="E127">
+        <v>-6.7</v>
+      </c>
+      <c r="F127">
+        <v>-7</v>
+      </c>
+      <c r="I127">
+        <v>2</v>
+      </c>
+      <c r="J127">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>13</v>
       </c>
       <c r="B128" s="2">
         <v>45873</v>
       </c>
-    </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C128" s="3">
+        <v>0.438194444444444</v>
+      </c>
+      <c r="D128">
+        <v>24.3</v>
+      </c>
+      <c r="E128">
+        <v>-6.8</v>
+      </c>
+      <c r="F128">
+        <v>-7</v>
+      </c>
+      <c r="I128">
+        <v>2</v>
+      </c>
+      <c r="J128">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>14</v>
       </c>
       <c r="B129" s="2">
         <v>45873</v>
       </c>
-    </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C129" s="3">
+        <v>0.44236111111111115</v>
+      </c>
+      <c r="D129">
+        <v>24.3</v>
+      </c>
+      <c r="E129">
+        <v>-7</v>
+      </c>
+      <c r="F129">
+        <v>-7.2</v>
+      </c>
+      <c r="G129">
+        <v>-7.2</v>
+      </c>
+      <c r="H129">
+        <v>-7.5</v>
+      </c>
+      <c r="I129">
+        <v>2</v>
+      </c>
+      <c r="J129">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>15</v>
       </c>
       <c r="B130" s="2">
         <v>45873</v>
       </c>
-    </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C130" s="3">
+        <v>0.4458333333333333</v>
+      </c>
+      <c r="D130">
+        <v>24.5</v>
+      </c>
+      <c r="E130">
+        <v>-7</v>
+      </c>
+      <c r="F130">
+        <v>-7.5</v>
+      </c>
+      <c r="G130">
+        <v>-7</v>
+      </c>
+      <c r="H130">
+        <v>-7.5</v>
+      </c>
+      <c r="I130">
+        <v>2</v>
+      </c>
+      <c r="J130">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>16</v>
       </c>
       <c r="B131" s="2">
         <v>45873</v>
       </c>
-    </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C131" s="3">
+        <v>0.44861111111111113</v>
+      </c>
+      <c r="D131">
+        <v>24.8</v>
+      </c>
+      <c r="E131">
+        <v>-6.4</v>
+      </c>
+      <c r="F131">
+        <v>-6.5</v>
+      </c>
+      <c r="I131">
+        <v>2</v>
+      </c>
+      <c r="J131">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>17</v>
       </c>
       <c r="B132" s="2">
         <v>45873</v>
       </c>
-    </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C132" s="3">
+        <v>0.45347222222222222</v>
+      </c>
+      <c r="D132">
+        <v>23.8</v>
+      </c>
+      <c r="E132">
+        <v>-6.7</v>
+      </c>
+      <c r="F132">
+        <v>-7</v>
+      </c>
+      <c r="I132">
+        <v>2</v>
+      </c>
+      <c r="J132">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>18</v>
       </c>
       <c r="B133" s="2">
         <v>45873</v>
       </c>
-    </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C133" s="3">
+        <v>0.45694444444444443</v>
+      </c>
+      <c r="D133">
+        <v>23.9</v>
+      </c>
+      <c r="E133">
+        <v>-7.4</v>
+      </c>
+      <c r="F133">
+        <v>-7.5</v>
+      </c>
+      <c r="I133">
+        <v>2</v>
+      </c>
+      <c r="J133">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>19</v>
       </c>
       <c r="B134" s="2">
         <v>45873</v>
       </c>
-    </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C134" s="3">
+        <v>0.4604166666666667</v>
+      </c>
+      <c r="D134">
+        <v>24.5</v>
+      </c>
+      <c r="E134">
+        <v>-7.5</v>
+      </c>
+      <c r="F134">
+        <v>-7.4</v>
+      </c>
+      <c r="I134">
+        <v>2</v>
+      </c>
+      <c r="J134">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>20</v>
       </c>
       <c r="B135" s="2">
         <v>45873</v>
       </c>
-    </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C135" s="3">
+        <v>0.46388888888888885</v>
+      </c>
+      <c r="D135">
+        <v>25.3</v>
+      </c>
+      <c r="E135">
+        <v>-7.8</v>
+      </c>
+      <c r="F135">
+        <v>-8</v>
+      </c>
+      <c r="I135">
+        <v>2</v>
+      </c>
+      <c r="J135">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>21</v>
       </c>
       <c r="B136" s="2">
         <v>45873</v>
+      </c>
+      <c r="C136" s="3">
+        <v>0.46736111111111112</v>
+      </c>
+      <c r="D136">
+        <v>25.4</v>
+      </c>
+      <c r="E136">
+        <v>-7.8</v>
+      </c>
+      <c r="F136">
+        <v>-7.8</v>
+      </c>
+      <c r="G136">
+        <v>-7.8</v>
+      </c>
+      <c r="H136">
+        <v>-8</v>
+      </c>
+      <c r="I136">
+        <v>2</v>
+      </c>
+      <c r="J136">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data updated till 25 Aug 2025 - preliminary seasonal emissions
</commit_message>
<xml_diff>
--- a/Field_Data/Field_Data.xlsx
+++ b/Field_Data/Field_Data.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11265"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11268"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="25">
   <si>
     <t>Plot</t>
   </si>
@@ -422,19 +422,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J136"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J181"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="8" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.5703125" customWidth="1"/>
-    <col min="10" max="10" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="8" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.5546875" customWidth="1"/>
+    <col min="10" max="10" width="13.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -466,7 +466,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -498,7 +498,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -521,7 +521,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -544,7 +544,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -567,7 +567,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -599,7 +599,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -622,7 +622,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -645,7 +645,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -677,7 +677,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -709,7 +709,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -732,7 +732,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -764,7 +764,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>18</v>
       </c>
@@ -796,7 +796,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -822,7 +822,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -854,7 +854,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -886,7 +886,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>7</v>
       </c>
@@ -909,7 +909,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -932,7 +932,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>9</v>
       </c>
@@ -955,7 +955,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>10</v>
       </c>
@@ -978,7 +978,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>11</v>
       </c>
@@ -1001,7 +1001,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>12</v>
       </c>
@@ -1033,7 +1033,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>13</v>
       </c>
@@ -1056,7 +1056,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>14</v>
       </c>
@@ -1088,7 +1088,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>15</v>
       </c>
@@ -1111,7 +1111,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>16</v>
       </c>
@@ -1143,7 +1143,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>17</v>
       </c>
@@ -1166,7 +1166,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>18</v>
       </c>
@@ -1189,7 +1189,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>19</v>
       </c>
@@ -1212,7 +1212,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>20</v>
       </c>
@@ -1235,7 +1235,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>21</v>
       </c>
@@ -1258,7 +1258,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>7</v>
       </c>
@@ -1281,7 +1281,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>8</v>
       </c>
@@ -1304,7 +1304,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>9</v>
       </c>
@@ -1327,7 +1327,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>10</v>
       </c>
@@ -1350,7 +1350,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>11</v>
       </c>
@@ -1373,7 +1373,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>12</v>
       </c>
@@ -1399,7 +1399,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>13</v>
       </c>
@@ -1431,7 +1431,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>14</v>
       </c>
@@ -1454,7 +1454,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>15</v>
       </c>
@@ -1486,7 +1486,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>16</v>
       </c>
@@ -1509,7 +1509,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>17</v>
       </c>
@@ -1532,7 +1532,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>18</v>
       </c>
@@ -1555,7 +1555,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>19</v>
       </c>
@@ -1578,7 +1578,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>20</v>
       </c>
@@ -1601,7 +1601,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>21</v>
       </c>
@@ -1624,7 +1624,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>7</v>
       </c>
@@ -1647,7 +1647,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>8</v>
       </c>
@@ -1670,7 +1670,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>9</v>
       </c>
@@ -1693,7 +1693,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>10</v>
       </c>
@@ -1716,7 +1716,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>11</v>
       </c>
@@ -1748,7 +1748,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>12</v>
       </c>
@@ -1780,7 +1780,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>13</v>
       </c>
@@ -1803,7 +1803,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>14</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>15</v>
       </c>
@@ -1858,7 +1858,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>16</v>
       </c>
@@ -1890,7 +1890,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>17</v>
       </c>
@@ -1913,7 +1913,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>18</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>19</v>
       </c>
@@ -1959,7 +1959,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>20</v>
       </c>
@@ -1991,7 +1991,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>21</v>
       </c>
@@ -2014,7 +2014,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>7</v>
       </c>
@@ -2046,7 +2046,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>8</v>
       </c>
@@ -2072,7 +2072,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>9</v>
       </c>
@@ -2104,7 +2104,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>10</v>
       </c>
@@ -2136,7 +2136,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>11</v>
       </c>
@@ -2159,7 +2159,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>12</v>
       </c>
@@ -2182,7 +2182,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>13</v>
       </c>
@@ -2205,7 +2205,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>14</v>
       </c>
@@ -2228,7 +2228,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>15</v>
       </c>
@@ -2251,7 +2251,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>16</v>
       </c>
@@ -2274,7 +2274,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>17</v>
       </c>
@@ -2297,7 +2297,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>18</v>
       </c>
@@ -2329,7 +2329,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>19</v>
       </c>
@@ -2352,7 +2352,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>20</v>
       </c>
@@ -2378,7 +2378,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>21</v>
       </c>
@@ -2401,7 +2401,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>7</v>
       </c>
@@ -2424,7 +2424,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -2447,7 +2447,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>9</v>
       </c>
@@ -2479,7 +2479,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>10</v>
       </c>
@@ -2511,7 +2511,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>11</v>
       </c>
@@ -2543,7 +2543,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>12</v>
       </c>
@@ -2566,7 +2566,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>13</v>
       </c>
@@ -2589,7 +2589,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>14</v>
       </c>
@@ -2621,7 +2621,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>15</v>
       </c>
@@ -2644,7 +2644,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>16</v>
       </c>
@@ -2676,7 +2676,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>17</v>
       </c>
@@ -2708,7 +2708,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>18</v>
       </c>
@@ -2740,7 +2740,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>19</v>
       </c>
@@ -2772,7 +2772,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>20</v>
       </c>
@@ -2795,7 +2795,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>21</v>
       </c>
@@ -2818,7 +2818,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>7</v>
       </c>
@@ -2841,7 +2841,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>8</v>
       </c>
@@ -2864,7 +2864,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>9</v>
       </c>
@@ -2887,7 +2887,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>10</v>
       </c>
@@ -2910,7 +2910,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>11</v>
       </c>
@@ -2933,7 +2933,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>12</v>
       </c>
@@ -2965,7 +2965,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>13</v>
       </c>
@@ -2997,7 +2997,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>14</v>
       </c>
@@ -3023,7 +3023,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>15</v>
       </c>
@@ -3046,7 +3046,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>16</v>
       </c>
@@ -3069,7 +3069,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>17</v>
       </c>
@@ -3101,7 +3101,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>18</v>
       </c>
@@ -3124,7 +3124,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>19</v>
       </c>
@@ -3147,7 +3147,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>20</v>
       </c>
@@ -3170,7 +3170,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>21</v>
       </c>
@@ -3202,7 +3202,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>7</v>
       </c>
@@ -3234,7 +3234,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>8</v>
       </c>
@@ -3257,7 +3257,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>9</v>
       </c>
@@ -3280,7 +3280,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>10</v>
       </c>
@@ -3303,7 +3303,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>11</v>
       </c>
@@ -3335,7 +3335,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>12</v>
       </c>
@@ -3358,7 +3358,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>13</v>
       </c>
@@ -3390,7 +3390,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>14</v>
       </c>
@@ -3416,7 +3416,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>15</v>
       </c>
@@ -3439,7 +3439,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>16</v>
       </c>
@@ -3462,7 +3462,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>17</v>
       </c>
@@ -3485,7 +3485,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>18</v>
       </c>
@@ -3508,7 +3508,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>19</v>
       </c>
@@ -3540,7 +3540,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>20</v>
       </c>
@@ -3566,7 +3566,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>21</v>
       </c>
@@ -3589,7 +3589,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>7</v>
       </c>
@@ -3615,7 +3615,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>8</v>
       </c>
@@ -3647,7 +3647,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>9</v>
       </c>
@@ -3670,7 +3670,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>10</v>
       </c>
@@ -3702,7 +3702,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>11</v>
       </c>
@@ -3734,7 +3734,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>12</v>
       </c>
@@ -3760,7 +3760,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>13</v>
       </c>
@@ -3786,7 +3786,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>14</v>
       </c>
@@ -3818,7 +3818,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>15</v>
       </c>
@@ -3850,7 +3850,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>16</v>
       </c>
@@ -3876,7 +3876,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>17</v>
       </c>
@@ -3902,7 +3902,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>18</v>
       </c>
@@ -3928,7 +3928,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>19</v>
       </c>
@@ -3954,7 +3954,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>20</v>
       </c>
@@ -3980,7 +3980,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>21</v>
       </c>
@@ -4009,6 +4009,1125 @@
         <v>2</v>
       </c>
       <c r="J136">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="137" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A137" t="s">
+        <v>7</v>
+      </c>
+      <c r="B137" s="2">
+        <v>45880</v>
+      </c>
+      <c r="C137" s="3">
+        <v>0.39027777777777778</v>
+      </c>
+      <c r="D137">
+        <v>24.7</v>
+      </c>
+      <c r="E137">
+        <v>-7</v>
+      </c>
+      <c r="I137">
+        <v>2.5</v>
+      </c>
+      <c r="J137">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="138" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A138" t="s">
+        <v>8</v>
+      </c>
+      <c r="B138" s="2">
+        <v>45880</v>
+      </c>
+      <c r="C138" s="3">
+        <v>0.39374999999999999</v>
+      </c>
+      <c r="D138">
+        <v>26.8</v>
+      </c>
+      <c r="E138">
+        <v>-7</v>
+      </c>
+      <c r="I138">
+        <v>2.5</v>
+      </c>
+      <c r="J138">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="139" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A139" t="s">
+        <v>9</v>
+      </c>
+      <c r="B139" s="2">
+        <v>45880</v>
+      </c>
+      <c r="C139" s="3">
+        <v>0.39722222222222198</v>
+      </c>
+      <c r="D139">
+        <v>26.9</v>
+      </c>
+      <c r="E139">
+        <v>-6.5</v>
+      </c>
+      <c r="I139">
+        <v>2.5</v>
+      </c>
+      <c r="J139">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="140" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A140" t="s">
+        <v>10</v>
+      </c>
+      <c r="B140" s="2">
+        <v>45880</v>
+      </c>
+      <c r="C140" s="3">
+        <v>0.39999999999999997</v>
+      </c>
+      <c r="D140">
+        <v>27.3</v>
+      </c>
+      <c r="E140">
+        <v>-6.5</v>
+      </c>
+      <c r="I140">
+        <v>2.5</v>
+      </c>
+      <c r="J140">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="141" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A141" t="s">
+        <v>11</v>
+      </c>
+      <c r="B141" s="2">
+        <v>45880</v>
+      </c>
+      <c r="C141" s="3">
+        <v>0.40347222222222223</v>
+      </c>
+      <c r="D141">
+        <v>26.3</v>
+      </c>
+      <c r="E141">
+        <v>-7</v>
+      </c>
+      <c r="I141">
+        <v>2.5</v>
+      </c>
+      <c r="J141">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="142" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A142" t="s">
+        <v>12</v>
+      </c>
+      <c r="B142" s="2">
+        <v>45880</v>
+      </c>
+      <c r="C142" s="3">
+        <v>0.406944444444444</v>
+      </c>
+      <c r="D142">
+        <v>26.6</v>
+      </c>
+      <c r="E142">
+        <v>-6.5</v>
+      </c>
+      <c r="I142">
+        <v>2.5</v>
+      </c>
+      <c r="J142">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="143" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A143" t="s">
+        <v>13</v>
+      </c>
+      <c r="B143" s="2">
+        <v>45880</v>
+      </c>
+      <c r="C143" s="3">
+        <v>0.41041666666666698</v>
+      </c>
+      <c r="D143">
+        <v>26.1</v>
+      </c>
+      <c r="E143">
+        <v>-7</v>
+      </c>
+      <c r="I143">
+        <v>2.5</v>
+      </c>
+      <c r="J143">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="144" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A144" t="s">
+        <v>14</v>
+      </c>
+      <c r="B144" s="2">
+        <v>45880</v>
+      </c>
+      <c r="C144" s="3">
+        <v>0.41388888888888897</v>
+      </c>
+      <c r="D144">
+        <v>26.7</v>
+      </c>
+      <c r="E144">
+        <v>-7</v>
+      </c>
+      <c r="I144">
+        <v>2.5</v>
+      </c>
+      <c r="J144">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="145" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A145" t="s">
+        <v>15</v>
+      </c>
+      <c r="B145" s="2">
+        <v>45880</v>
+      </c>
+      <c r="C145" s="3">
+        <v>0.41736111111111102</v>
+      </c>
+      <c r="D145">
+        <v>25.6</v>
+      </c>
+      <c r="E145">
+        <v>-7.5</v>
+      </c>
+      <c r="I145">
+        <v>2.5</v>
+      </c>
+      <c r="J145">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="146" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A146" t="s">
+        <v>16</v>
+      </c>
+      <c r="B146" s="2">
+        <v>45880</v>
+      </c>
+      <c r="C146" s="3">
+        <v>0.420833333333334</v>
+      </c>
+      <c r="D146">
+        <v>26.6</v>
+      </c>
+      <c r="E146">
+        <v>-6.5</v>
+      </c>
+      <c r="F146">
+        <v>-6.7</v>
+      </c>
+      <c r="G146">
+        <v>-6.7</v>
+      </c>
+      <c r="H146">
+        <v>-6.7</v>
+      </c>
+      <c r="I146">
+        <v>2.5</v>
+      </c>
+      <c r="J146">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="147" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A147" t="s">
+        <v>17</v>
+      </c>
+      <c r="B147" s="2">
+        <v>45880</v>
+      </c>
+      <c r="C147" s="3">
+        <v>0.42430555555555599</v>
+      </c>
+      <c r="D147">
+        <v>26.5</v>
+      </c>
+      <c r="E147">
+        <v>-7</v>
+      </c>
+      <c r="F147">
+        <v>-6.5</v>
+      </c>
+      <c r="G147">
+        <v>-6</v>
+      </c>
+      <c r="H147">
+        <v>-6.3</v>
+      </c>
+      <c r="I147">
+        <v>2.5</v>
+      </c>
+      <c r="J147">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="148" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A148" t="s">
+        <v>18</v>
+      </c>
+      <c r="B148" s="2">
+        <v>45880</v>
+      </c>
+      <c r="C148" s="3">
+        <v>0.42777777777777798</v>
+      </c>
+      <c r="D148">
+        <v>25.8</v>
+      </c>
+      <c r="E148">
+        <v>-7</v>
+      </c>
+      <c r="I148">
+        <v>2.5</v>
+      </c>
+      <c r="J148">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="149" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A149" t="s">
+        <v>19</v>
+      </c>
+      <c r="B149" s="2">
+        <v>45880</v>
+      </c>
+      <c r="C149" s="3">
+        <v>0.43125000000000002</v>
+      </c>
+      <c r="D149">
+        <v>25.3</v>
+      </c>
+      <c r="E149">
+        <v>-7.5</v>
+      </c>
+      <c r="F149">
+        <v>-8</v>
+      </c>
+      <c r="G149">
+        <v>-8</v>
+      </c>
+      <c r="H149">
+        <v>-8</v>
+      </c>
+      <c r="I149">
+        <v>2.5</v>
+      </c>
+      <c r="J149">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="150" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A150" t="s">
+        <v>20</v>
+      </c>
+      <c r="B150" s="2">
+        <v>45880</v>
+      </c>
+      <c r="C150" s="3">
+        <v>0.43472222222222301</v>
+      </c>
+      <c r="D150">
+        <v>25.9</v>
+      </c>
+      <c r="E150">
+        <v>-7.5</v>
+      </c>
+      <c r="I150">
+        <v>2.5</v>
+      </c>
+      <c r="J150">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="151" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A151" t="s">
+        <v>21</v>
+      </c>
+      <c r="B151" s="2">
+        <v>45880</v>
+      </c>
+      <c r="C151" s="3">
+        <v>0.438194444444445</v>
+      </c>
+      <c r="D151">
+        <v>26.4</v>
+      </c>
+      <c r="E151">
+        <v>-7</v>
+      </c>
+      <c r="I151">
+        <v>2.5</v>
+      </c>
+      <c r="J151">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="152" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A152" t="s">
+        <v>7</v>
+      </c>
+      <c r="B152" s="2">
+        <v>45887</v>
+      </c>
+      <c r="C152" s="3">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="D152">
+        <v>23.4</v>
+      </c>
+      <c r="E152">
+        <v>-7.8</v>
+      </c>
+      <c r="I152">
+        <v>2.5</v>
+      </c>
+      <c r="J152">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="153" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A153" t="s">
+        <v>8</v>
+      </c>
+      <c r="B153" s="2">
+        <v>45887</v>
+      </c>
+      <c r="C153" s="3">
+        <v>0.39999999999999997</v>
+      </c>
+      <c r="D153">
+        <v>23.4</v>
+      </c>
+      <c r="E153">
+        <v>-7.5</v>
+      </c>
+      <c r="I153">
+        <v>2.5</v>
+      </c>
+      <c r="J153">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="154" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A154" t="s">
+        <v>9</v>
+      </c>
+      <c r="B154" s="2">
+        <v>45887</v>
+      </c>
+      <c r="C154" s="3">
+        <v>0.40486111111111112</v>
+      </c>
+      <c r="D154">
+        <v>22.8</v>
+      </c>
+      <c r="E154">
+        <v>-7.5</v>
+      </c>
+      <c r="I154">
+        <v>2.5</v>
+      </c>
+      <c r="J154">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="155" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A155" t="s">
+        <v>10</v>
+      </c>
+      <c r="B155" s="2">
+        <v>45887</v>
+      </c>
+      <c r="C155" s="3">
+        <v>0.40902777777777777</v>
+      </c>
+      <c r="D155">
+        <v>22.4</v>
+      </c>
+      <c r="E155">
+        <v>-7.5</v>
+      </c>
+      <c r="I155">
+        <v>2.5</v>
+      </c>
+      <c r="J155">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="156" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A156" t="s">
+        <v>11</v>
+      </c>
+      <c r="B156" s="2">
+        <v>45887</v>
+      </c>
+      <c r="C156" s="3">
+        <v>0.41319444444444442</v>
+      </c>
+      <c r="D156">
+        <v>22.4</v>
+      </c>
+      <c r="E156">
+        <v>-7.4</v>
+      </c>
+      <c r="I156">
+        <v>2.5</v>
+      </c>
+      <c r="J156">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="157" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A157" t="s">
+        <v>12</v>
+      </c>
+      <c r="B157" s="2">
+        <v>45887</v>
+      </c>
+      <c r="C157" s="3">
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="D157">
+        <v>23.4</v>
+      </c>
+      <c r="E157">
+        <v>-7.6</v>
+      </c>
+      <c r="F157">
+        <v>-7.8</v>
+      </c>
+      <c r="G157">
+        <v>-7.9</v>
+      </c>
+      <c r="H157">
+        <v>-7.9</v>
+      </c>
+      <c r="I157">
+        <v>2.5</v>
+      </c>
+      <c r="J157">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="158" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A158" t="s">
+        <v>13</v>
+      </c>
+      <c r="B158" s="2">
+        <v>45887</v>
+      </c>
+      <c r="C158" s="3">
+        <v>0.43194444444444446</v>
+      </c>
+      <c r="D158">
+        <v>23.4</v>
+      </c>
+      <c r="E158">
+        <v>-7.7</v>
+      </c>
+      <c r="F158">
+        <v>-7.5</v>
+      </c>
+      <c r="G158">
+        <v>-7.9</v>
+      </c>
+      <c r="H158">
+        <v>-7.6</v>
+      </c>
+      <c r="I158">
+        <v>2.5</v>
+      </c>
+      <c r="J158">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="159" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A159" t="s">
+        <v>14</v>
+      </c>
+      <c r="B159" s="2">
+        <v>45887</v>
+      </c>
+      <c r="C159" s="3">
+        <v>0.4368055555555555</v>
+      </c>
+      <c r="D159">
+        <v>23.4</v>
+      </c>
+      <c r="E159">
+        <v>-8</v>
+      </c>
+      <c r="I159">
+        <v>2.5</v>
+      </c>
+      <c r="J159">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="160" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A160" t="s">
+        <v>15</v>
+      </c>
+      <c r="B160" s="2">
+        <v>45887</v>
+      </c>
+      <c r="C160" s="3">
+        <v>0.44097222222222227</v>
+      </c>
+      <c r="D160">
+        <v>23.4</v>
+      </c>
+      <c r="E160">
+        <v>-8.1</v>
+      </c>
+      <c r="I160">
+        <v>2.5</v>
+      </c>
+      <c r="J160">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="161" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A161" t="s">
+        <v>16</v>
+      </c>
+      <c r="B161" s="2">
+        <v>45887</v>
+      </c>
+      <c r="C161" s="3">
+        <v>0.44513888888888892</v>
+      </c>
+      <c r="D161">
+        <v>23.4</v>
+      </c>
+      <c r="E161">
+        <v>-7.5</v>
+      </c>
+      <c r="I161">
+        <v>2.5</v>
+      </c>
+      <c r="J161">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="162" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A162" t="s">
+        <v>17</v>
+      </c>
+      <c r="B162" s="2">
+        <v>45887</v>
+      </c>
+      <c r="C162" s="3">
+        <v>0.45</v>
+      </c>
+      <c r="D162">
+        <v>23.4</v>
+      </c>
+      <c r="E162">
+        <v>-7.8</v>
+      </c>
+      <c r="I162">
+        <v>2.5</v>
+      </c>
+      <c r="J162">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="163" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A163" t="s">
+        <v>18</v>
+      </c>
+      <c r="B163" s="2">
+        <v>45887</v>
+      </c>
+      <c r="C163" s="3">
+        <v>0.45555555555555555</v>
+      </c>
+      <c r="D163">
+        <v>23.4</v>
+      </c>
+      <c r="E163">
+        <v>-8</v>
+      </c>
+      <c r="F163">
+        <v>-8.3000000000000007</v>
+      </c>
+      <c r="G163">
+        <v>-8.3000000000000007</v>
+      </c>
+      <c r="H163">
+        <v>-8.5</v>
+      </c>
+      <c r="I163">
+        <v>2.5</v>
+      </c>
+      <c r="J163">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="164" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A164" t="s">
+        <v>19</v>
+      </c>
+      <c r="B164" s="2">
+        <v>45887</v>
+      </c>
+      <c r="C164" s="3">
+        <v>0.4597222222222222</v>
+      </c>
+      <c r="D164">
+        <v>23.4</v>
+      </c>
+      <c r="E164">
+        <v>-8.5</v>
+      </c>
+      <c r="I164">
+        <v>2.5</v>
+      </c>
+      <c r="J164">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="165" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A165" t="s">
+        <v>20</v>
+      </c>
+      <c r="B165" s="2">
+        <v>45887</v>
+      </c>
+      <c r="C165" s="3">
+        <v>0.46388888888888885</v>
+      </c>
+      <c r="D165">
+        <v>23.4</v>
+      </c>
+      <c r="E165">
+        <v>-8.8000000000000007</v>
+      </c>
+      <c r="I165">
+        <v>2.5</v>
+      </c>
+      <c r="J165">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="166" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A166" t="s">
+        <v>21</v>
+      </c>
+      <c r="B166" s="2">
+        <v>45887</v>
+      </c>
+      <c r="C166" s="3">
+        <v>0.4680555555555555</v>
+      </c>
+      <c r="D166">
+        <v>23.4</v>
+      </c>
+      <c r="E166">
+        <v>-8.5</v>
+      </c>
+      <c r="I166">
+        <v>2.5</v>
+      </c>
+      <c r="J166">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="167" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A167" t="s">
+        <v>7</v>
+      </c>
+      <c r="B167" s="2">
+        <v>45894</v>
+      </c>
+      <c r="C167" s="3">
+        <v>0.3979166666666667</v>
+      </c>
+      <c r="D167">
+        <v>25.9</v>
+      </c>
+      <c r="E167">
+        <v>-7.7</v>
+      </c>
+      <c r="I167">
+        <v>3</v>
+      </c>
+      <c r="J167">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="168" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A168" t="s">
+        <v>8</v>
+      </c>
+      <c r="B168" s="2">
+        <v>45894</v>
+      </c>
+      <c r="C168" s="3">
+        <v>0.40138888888888885</v>
+      </c>
+      <c r="D168">
+        <v>27.4</v>
+      </c>
+      <c r="E168">
+        <v>-7</v>
+      </c>
+      <c r="I168">
+        <v>3</v>
+      </c>
+      <c r="J168">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="169" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A169" t="s">
+        <v>9</v>
+      </c>
+      <c r="B169" s="2">
+        <v>45894</v>
+      </c>
+      <c r="C169" s="3">
+        <v>0.40486111111111101</v>
+      </c>
+      <c r="D169">
+        <v>26.7</v>
+      </c>
+      <c r="E169">
+        <v>-7</v>
+      </c>
+      <c r="I169">
+        <v>3</v>
+      </c>
+      <c r="J169">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="170" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A170" t="s">
+        <v>10</v>
+      </c>
+      <c r="B170" s="2">
+        <v>45894</v>
+      </c>
+      <c r="C170" s="3">
+        <v>0.40833333333333299</v>
+      </c>
+      <c r="D170">
+        <v>27</v>
+      </c>
+      <c r="E170">
+        <v>-7</v>
+      </c>
+      <c r="F170">
+        <v>-7.2</v>
+      </c>
+      <c r="G170">
+        <v>-7.2</v>
+      </c>
+      <c r="H170">
+        <v>-7.2</v>
+      </c>
+      <c r="I170">
+        <v>3</v>
+      </c>
+      <c r="J170">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="171" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A171" t="s">
+        <v>11</v>
+      </c>
+      <c r="B171" s="2">
+        <v>45894</v>
+      </c>
+      <c r="C171" s="3">
+        <v>0.41180555555555498</v>
+      </c>
+      <c r="D171">
+        <v>27</v>
+      </c>
+      <c r="E171">
+        <v>-7.5</v>
+      </c>
+      <c r="I171">
+        <v>3</v>
+      </c>
+      <c r="J171">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="172" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A172" t="s">
+        <v>12</v>
+      </c>
+      <c r="B172" s="2">
+        <v>45894</v>
+      </c>
+      <c r="C172" s="3">
+        <v>0.4152777777777778</v>
+      </c>
+      <c r="D172">
+        <v>28</v>
+      </c>
+      <c r="E172">
+        <v>-7.2</v>
+      </c>
+      <c r="F172">
+        <v>-7.2</v>
+      </c>
+      <c r="I172">
+        <v>3</v>
+      </c>
+      <c r="J172">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="173" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A173" t="s">
+        <v>13</v>
+      </c>
+      <c r="B173" s="2">
+        <v>45894</v>
+      </c>
+      <c r="C173" s="3">
+        <v>0.41875000000000001</v>
+      </c>
+      <c r="D173">
+        <v>26.3</v>
+      </c>
+      <c r="E173">
+        <v>-7.7</v>
+      </c>
+      <c r="F173">
+        <v>-8</v>
+      </c>
+      <c r="G173">
+        <v>-7.8</v>
+      </c>
+      <c r="H173">
+        <v>-7.7</v>
+      </c>
+      <c r="I173">
+        <v>3</v>
+      </c>
+      <c r="J173">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="174" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A174" t="s">
+        <v>14</v>
+      </c>
+      <c r="B174" s="2">
+        <v>45894</v>
+      </c>
+      <c r="C174" s="3">
+        <v>0.422222222222222</v>
+      </c>
+      <c r="D174">
+        <v>27.7</v>
+      </c>
+      <c r="E174">
+        <v>-7.5</v>
+      </c>
+      <c r="F174">
+        <v>-7.5</v>
+      </c>
+      <c r="G174">
+        <v>-7.8</v>
+      </c>
+      <c r="H174">
+        <v>-7.3</v>
+      </c>
+      <c r="I174">
+        <v>3</v>
+      </c>
+      <c r="J174">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="175" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A175" t="s">
+        <v>15</v>
+      </c>
+      <c r="B175" s="2">
+        <v>45894</v>
+      </c>
+      <c r="C175" s="3">
+        <v>0.42569444444444399</v>
+      </c>
+      <c r="D175">
+        <v>27</v>
+      </c>
+      <c r="E175">
+        <v>-8.1999999999999993</v>
+      </c>
+      <c r="I175">
+        <v>3</v>
+      </c>
+      <c r="J175">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="176" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A176" t="s">
+        <v>16</v>
+      </c>
+      <c r="B176" s="2">
+        <v>45894</v>
+      </c>
+      <c r="C176" s="3">
+        <v>0.42916666666666597</v>
+      </c>
+      <c r="D176">
+        <v>28.3</v>
+      </c>
+      <c r="E176">
+        <v>-7.2</v>
+      </c>
+      <c r="I176">
+        <v>3</v>
+      </c>
+      <c r="J176">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="177" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A177" t="s">
+        <v>17</v>
+      </c>
+      <c r="B177" s="2">
+        <v>45894</v>
+      </c>
+      <c r="C177" s="3">
+        <v>0.43263888888888802</v>
+      </c>
+      <c r="D177">
+        <v>27.7</v>
+      </c>
+      <c r="E177">
+        <v>-7</v>
+      </c>
+      <c r="I177">
+        <v>3</v>
+      </c>
+      <c r="J177">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="178" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A178" t="s">
+        <v>18</v>
+      </c>
+      <c r="B178" s="2">
+        <v>45894</v>
+      </c>
+      <c r="C178" s="3">
+        <v>0.43611111111111001</v>
+      </c>
+      <c r="D178">
+        <v>28.8</v>
+      </c>
+      <c r="E178">
+        <v>-9</v>
+      </c>
+      <c r="I178">
+        <v>3</v>
+      </c>
+      <c r="J178">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="179" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A179" t="s">
+        <v>19</v>
+      </c>
+      <c r="B179" s="2">
+        <v>45894</v>
+      </c>
+      <c r="C179" s="3">
+        <v>0.43958333333333299</v>
+      </c>
+      <c r="D179">
+        <v>26.9</v>
+      </c>
+      <c r="E179">
+        <v>-8.8000000000000007</v>
+      </c>
+      <c r="I179">
+        <v>3</v>
+      </c>
+      <c r="J179">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="180" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A180" t="s">
+        <v>20</v>
+      </c>
+      <c r="B180" s="2">
+        <v>45894</v>
+      </c>
+      <c r="C180" s="3">
+        <v>0.44305555555555498</v>
+      </c>
+      <c r="D180">
+        <v>27.6</v>
+      </c>
+      <c r="E180">
+        <v>-8.1999999999999993</v>
+      </c>
+      <c r="I180">
+        <v>3</v>
+      </c>
+      <c r="J180">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="181" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A181" t="s">
+        <v>21</v>
+      </c>
+      <c r="B181" s="2">
+        <v>45894</v>
+      </c>
+      <c r="C181" s="3">
+        <v>0.44652777777777702</v>
+      </c>
+      <c r="D181">
+        <v>27</v>
+      </c>
+      <c r="E181">
+        <v>-8</v>
+      </c>
+      <c r="I181">
+        <v>3</v>
+      </c>
+      <c r="J181">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added final yield raw data, keyed in all field data for licor measurements
</commit_message>
<xml_diff>
--- a/Field_Data/Field_Data.xlsx
+++ b/Field_Data/Field_Data.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11268"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11265"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="25">
   <si>
     <t>Plot</t>
   </si>
@@ -422,19 +422,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J196"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J256"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="8" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.5546875" customWidth="1"/>
-    <col min="10" max="10" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="8" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.5703125" customWidth="1"/>
+    <col min="10" max="10" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -466,7 +466,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -498,7 +498,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -521,7 +521,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -544,7 +544,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -567,7 +567,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -599,7 +599,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -622,7 +622,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -645,7 +645,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -677,7 +677,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -709,7 +709,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -732,7 +732,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -764,7 +764,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>18</v>
       </c>
@@ -796,7 +796,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -822,7 +822,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -854,7 +854,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -886,7 +886,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>7</v>
       </c>
@@ -909,7 +909,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -932,7 +932,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>9</v>
       </c>
@@ -955,7 +955,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>10</v>
       </c>
@@ -978,7 +978,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>11</v>
       </c>
@@ -1001,7 +1001,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>12</v>
       </c>
@@ -1033,7 +1033,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>13</v>
       </c>
@@ -1056,7 +1056,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>14</v>
       </c>
@@ -1088,7 +1088,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>15</v>
       </c>
@@ -1111,7 +1111,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>16</v>
       </c>
@@ -1143,7 +1143,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>17</v>
       </c>
@@ -1166,7 +1166,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>18</v>
       </c>
@@ -1189,7 +1189,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>19</v>
       </c>
@@ -1212,7 +1212,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>20</v>
       </c>
@@ -1235,7 +1235,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>21</v>
       </c>
@@ -1258,7 +1258,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>7</v>
       </c>
@@ -1281,7 +1281,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>8</v>
       </c>
@@ -1304,7 +1304,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>9</v>
       </c>
@@ -1327,7 +1327,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>10</v>
       </c>
@@ -1350,7 +1350,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>11</v>
       </c>
@@ -1373,7 +1373,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>12</v>
       </c>
@@ -1399,7 +1399,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>13</v>
       </c>
@@ -1431,7 +1431,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>14</v>
       </c>
@@ -1454,7 +1454,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>15</v>
       </c>
@@ -1486,7 +1486,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>16</v>
       </c>
@@ -1509,7 +1509,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>17</v>
       </c>
@@ -1532,7 +1532,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>18</v>
       </c>
@@ -1555,7 +1555,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>19</v>
       </c>
@@ -1578,7 +1578,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>20</v>
       </c>
@@ -1601,7 +1601,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>21</v>
       </c>
@@ -1624,7 +1624,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>7</v>
       </c>
@@ -1647,7 +1647,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>8</v>
       </c>
@@ -1670,7 +1670,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>9</v>
       </c>
@@ -1693,7 +1693,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>10</v>
       </c>
@@ -1716,7 +1716,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>11</v>
       </c>
@@ -1748,7 +1748,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>12</v>
       </c>
@@ -1780,7 +1780,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>13</v>
       </c>
@@ -1803,7 +1803,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>14</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>15</v>
       </c>
@@ -1858,7 +1858,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>16</v>
       </c>
@@ -1890,7 +1890,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>17</v>
       </c>
@@ -1913,7 +1913,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>18</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>19</v>
       </c>
@@ -1959,7 +1959,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>20</v>
       </c>
@@ -1991,7 +1991,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>21</v>
       </c>
@@ -2014,7 +2014,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>7</v>
       </c>
@@ -2046,7 +2046,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>8</v>
       </c>
@@ -2072,7 +2072,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>9</v>
       </c>
@@ -2104,7 +2104,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>10</v>
       </c>
@@ -2136,7 +2136,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>11</v>
       </c>
@@ -2159,7 +2159,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>12</v>
       </c>
@@ -2182,7 +2182,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>13</v>
       </c>
@@ -2205,7 +2205,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>14</v>
       </c>
@@ -2228,7 +2228,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>15</v>
       </c>
@@ -2251,7 +2251,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>16</v>
       </c>
@@ -2274,7 +2274,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>17</v>
       </c>
@@ -2297,7 +2297,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>18</v>
       </c>
@@ -2329,7 +2329,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>19</v>
       </c>
@@ -2352,7 +2352,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>20</v>
       </c>
@@ -2378,7 +2378,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>21</v>
       </c>
@@ -2401,7 +2401,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>7</v>
       </c>
@@ -2424,7 +2424,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -2447,7 +2447,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>9</v>
       </c>
@@ -2479,7 +2479,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>10</v>
       </c>
@@ -2511,7 +2511,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>11</v>
       </c>
@@ -2543,7 +2543,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>12</v>
       </c>
@@ -2566,7 +2566,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>13</v>
       </c>
@@ -2589,7 +2589,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>14</v>
       </c>
@@ -2621,7 +2621,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>15</v>
       </c>
@@ -2644,7 +2644,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>16</v>
       </c>
@@ -2676,7 +2676,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>17</v>
       </c>
@@ -2708,7 +2708,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>18</v>
       </c>
@@ -2740,7 +2740,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>19</v>
       </c>
@@ -2772,7 +2772,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>20</v>
       </c>
@@ -2795,7 +2795,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>21</v>
       </c>
@@ -2818,7 +2818,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>7</v>
       </c>
@@ -2841,7 +2841,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>8</v>
       </c>
@@ -2864,7 +2864,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>9</v>
       </c>
@@ -2887,7 +2887,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>10</v>
       </c>
@@ -2910,7 +2910,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>11</v>
       </c>
@@ -2933,7 +2933,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>12</v>
       </c>
@@ -2965,7 +2965,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>13</v>
       </c>
@@ -2997,7 +2997,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>14</v>
       </c>
@@ -3023,7 +3023,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>15</v>
       </c>
@@ -3046,7 +3046,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>16</v>
       </c>
@@ -3069,7 +3069,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>17</v>
       </c>
@@ -3101,7 +3101,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>18</v>
       </c>
@@ -3124,7 +3124,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>19</v>
       </c>
@@ -3147,7 +3147,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>20</v>
       </c>
@@ -3170,7 +3170,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>21</v>
       </c>
@@ -3202,7 +3202,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>7</v>
       </c>
@@ -3234,7 +3234,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>8</v>
       </c>
@@ -3257,7 +3257,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>9</v>
       </c>
@@ -3280,7 +3280,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>10</v>
       </c>
@@ -3303,7 +3303,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>11</v>
       </c>
@@ -3335,7 +3335,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>12</v>
       </c>
@@ -3358,7 +3358,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>13</v>
       </c>
@@ -3390,7 +3390,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>14</v>
       </c>
@@ -3416,7 +3416,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>15</v>
       </c>
@@ -3439,7 +3439,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>16</v>
       </c>
@@ -3462,7 +3462,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>17</v>
       </c>
@@ -3485,7 +3485,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>18</v>
       </c>
@@ -3508,7 +3508,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>19</v>
       </c>
@@ -3540,7 +3540,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>20</v>
       </c>
@@ -3566,7 +3566,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>21</v>
       </c>
@@ -3589,7 +3589,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>7</v>
       </c>
@@ -3615,7 +3615,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>8</v>
       </c>
@@ -3647,7 +3647,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>9</v>
       </c>
@@ -3670,7 +3670,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>10</v>
       </c>
@@ -3702,7 +3702,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>11</v>
       </c>
@@ -3734,7 +3734,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>12</v>
       </c>
@@ -3760,7 +3760,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>13</v>
       </c>
@@ -3786,7 +3786,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>14</v>
       </c>
@@ -3818,7 +3818,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>15</v>
       </c>
@@ -3850,7 +3850,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>16</v>
       </c>
@@ -3876,7 +3876,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>17</v>
       </c>
@@ -3902,7 +3902,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>18</v>
       </c>
@@ -3928,7 +3928,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>19</v>
       </c>
@@ -3954,7 +3954,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>20</v>
       </c>
@@ -3980,7 +3980,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>21</v>
       </c>
@@ -4012,7 +4012,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>7</v>
       </c>
@@ -4035,7 +4035,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>8</v>
       </c>
@@ -4058,7 +4058,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>9</v>
       </c>
@@ -4081,7 +4081,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>10</v>
       </c>
@@ -4104,7 +4104,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>11</v>
       </c>
@@ -4127,7 +4127,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>12</v>
       </c>
@@ -4150,7 +4150,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>13</v>
       </c>
@@ -4173,7 +4173,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>14</v>
       </c>
@@ -4196,7 +4196,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>15</v>
       </c>
@@ -4219,7 +4219,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>16</v>
       </c>
@@ -4251,7 +4251,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>17</v>
       </c>
@@ -4283,7 +4283,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>18</v>
       </c>
@@ -4306,7 +4306,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>19</v>
       </c>
@@ -4338,7 +4338,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>20</v>
       </c>
@@ -4361,7 +4361,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>21</v>
       </c>
@@ -4384,7 +4384,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>7</v>
       </c>
@@ -4407,7 +4407,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>8</v>
       </c>
@@ -4430,7 +4430,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>9</v>
       </c>
@@ -4453,7 +4453,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>10</v>
       </c>
@@ -4476,7 +4476,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>11</v>
       </c>
@@ -4499,7 +4499,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>12</v>
       </c>
@@ -4531,7 +4531,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="158" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>13</v>
       </c>
@@ -4563,7 +4563,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="159" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>14</v>
       </c>
@@ -4586,7 +4586,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="160" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>15</v>
       </c>
@@ -4609,7 +4609,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="161" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>16</v>
       </c>
@@ -4632,7 +4632,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="162" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>17</v>
       </c>
@@ -4655,7 +4655,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="163" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>18</v>
       </c>
@@ -4687,7 +4687,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="164" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>19</v>
       </c>
@@ -4710,7 +4710,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="165" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>20</v>
       </c>
@@ -4733,7 +4733,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>21</v>
       </c>
@@ -4756,7 +4756,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="167" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>7</v>
       </c>
@@ -4779,7 +4779,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="168" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>8</v>
       </c>
@@ -4802,7 +4802,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="169" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>9</v>
       </c>
@@ -4825,7 +4825,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="170" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>10</v>
       </c>
@@ -4857,7 +4857,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="171" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>11</v>
       </c>
@@ -4880,7 +4880,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="172" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>12</v>
       </c>
@@ -4906,7 +4906,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="173" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>13</v>
       </c>
@@ -4938,7 +4938,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="174" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>14</v>
       </c>
@@ -4970,7 +4970,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="175" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>15</v>
       </c>
@@ -4993,7 +4993,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="176" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>16</v>
       </c>
@@ -5016,7 +5016,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="177" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>17</v>
       </c>
@@ -5039,7 +5039,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="178" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>18</v>
       </c>
@@ -5062,7 +5062,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="179" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>19</v>
       </c>
@@ -5085,7 +5085,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="180" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>20</v>
       </c>
@@ -5108,7 +5108,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="181" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>21</v>
       </c>
@@ -5131,7 +5131,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="182" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>7</v>
       </c>
@@ -5157,7 +5157,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="183" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>8</v>
       </c>
@@ -5183,7 +5183,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="184" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>9</v>
       </c>
@@ -5209,7 +5209,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="185" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>10</v>
       </c>
@@ -5232,7 +5232,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="186" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>11</v>
       </c>
@@ -5258,7 +5258,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="187" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>12</v>
       </c>
@@ -5284,7 +5284,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="188" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>13</v>
       </c>
@@ -5310,7 +5310,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="189" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>14</v>
       </c>
@@ -5342,7 +5342,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="190" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>15</v>
       </c>
@@ -5365,7 +5365,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="191" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>16</v>
       </c>
@@ -5388,7 +5388,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="192" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>17</v>
       </c>
@@ -5411,7 +5411,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="193" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>18</v>
       </c>
@@ -5443,7 +5443,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="194" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>19</v>
       </c>
@@ -5466,7 +5466,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="195" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>20</v>
       </c>
@@ -5489,7 +5489,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="196" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>21</v>
       </c>
@@ -5510,6 +5510,1431 @@
       </c>
       <c r="J196">
         <v>4</v>
+      </c>
+    </row>
+    <row r="197" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A197" t="s">
+        <v>7</v>
+      </c>
+      <c r="B197" s="2">
+        <v>45908</v>
+      </c>
+      <c r="C197" s="3">
+        <v>0.40069444444444446</v>
+      </c>
+      <c r="D197">
+        <v>22.8</v>
+      </c>
+      <c r="E197">
+        <v>2.5</v>
+      </c>
+      <c r="I197">
+        <v>2.5</v>
+      </c>
+      <c r="J197">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="198" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A198" t="s">
+        <v>8</v>
+      </c>
+      <c r="B198" s="2">
+        <v>45908</v>
+      </c>
+      <c r="C198" s="3">
+        <v>0.40416666666666662</v>
+      </c>
+      <c r="D198">
+        <v>23</v>
+      </c>
+      <c r="E198">
+        <v>2.75</v>
+      </c>
+      <c r="I198">
+        <v>2.5</v>
+      </c>
+      <c r="J198">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="199" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A199" t="s">
+        <v>9</v>
+      </c>
+      <c r="B199" s="2">
+        <v>45908</v>
+      </c>
+      <c r="C199" s="3">
+        <v>0.4069444444444445</v>
+      </c>
+      <c r="D199">
+        <v>23.1</v>
+      </c>
+      <c r="E199">
+        <v>3</v>
+      </c>
+      <c r="I199">
+        <v>2.5</v>
+      </c>
+      <c r="J199">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="200" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A200" t="s">
+        <v>10</v>
+      </c>
+      <c r="B200" s="2">
+        <v>45908</v>
+      </c>
+      <c r="C200" s="3">
+        <v>0.40972222222222227</v>
+      </c>
+      <c r="D200">
+        <v>23.9</v>
+      </c>
+      <c r="E200">
+        <v>2.9</v>
+      </c>
+      <c r="I200">
+        <v>2.5</v>
+      </c>
+      <c r="J200">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="201" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
+        <v>11</v>
+      </c>
+      <c r="B201" s="2">
+        <v>45908</v>
+      </c>
+      <c r="C201" s="3">
+        <v>0.41250000000000003</v>
+      </c>
+      <c r="D201">
+        <v>23.2</v>
+      </c>
+      <c r="E201">
+        <v>2.8</v>
+      </c>
+      <c r="I201">
+        <v>2.5</v>
+      </c>
+      <c r="J201">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="202" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
+        <v>12</v>
+      </c>
+      <c r="B202" s="2">
+        <v>45908</v>
+      </c>
+      <c r="C202" s="3">
+        <v>0.41597222222222219</v>
+      </c>
+      <c r="D202">
+        <v>23.3</v>
+      </c>
+      <c r="E202">
+        <v>2.5</v>
+      </c>
+      <c r="F202">
+        <v>2.4</v>
+      </c>
+      <c r="G202">
+        <v>2.4</v>
+      </c>
+      <c r="H202">
+        <v>2.6</v>
+      </c>
+      <c r="I202">
+        <v>2.5</v>
+      </c>
+      <c r="J202">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="203" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
+        <v>13</v>
+      </c>
+      <c r="B203" s="2">
+        <v>45908</v>
+      </c>
+      <c r="C203" s="3">
+        <v>0.41944444444444445</v>
+      </c>
+      <c r="D203">
+        <v>23.5</v>
+      </c>
+      <c r="E203">
+        <v>2.4</v>
+      </c>
+      <c r="I203">
+        <v>2.5</v>
+      </c>
+      <c r="J203">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="204" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A204" t="s">
+        <v>14</v>
+      </c>
+      <c r="B204" s="2">
+        <v>45908</v>
+      </c>
+      <c r="C204" s="3">
+        <v>0.42291666666666666</v>
+      </c>
+      <c r="D204">
+        <v>24.3</v>
+      </c>
+      <c r="E204">
+        <v>2.4</v>
+      </c>
+      <c r="I204">
+        <v>2.5</v>
+      </c>
+      <c r="J204">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="205" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A205" t="s">
+        <v>15</v>
+      </c>
+      <c r="B205" s="2">
+        <v>45908</v>
+      </c>
+      <c r="C205" s="3">
+        <v>0.42638888888888887</v>
+      </c>
+      <c r="D205">
+        <v>24.1</v>
+      </c>
+      <c r="E205">
+        <v>2.4</v>
+      </c>
+      <c r="I205">
+        <v>2.5</v>
+      </c>
+      <c r="J205">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="206" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A206" t="s">
+        <v>16</v>
+      </c>
+      <c r="B206" s="2">
+        <v>45908</v>
+      </c>
+      <c r="C206" s="3">
+        <v>0.4291666666666667</v>
+      </c>
+      <c r="D206">
+        <v>24.7</v>
+      </c>
+      <c r="E206">
+        <v>2.9</v>
+      </c>
+      <c r="I206">
+        <v>2.5</v>
+      </c>
+      <c r="J206">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="207" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A207" t="s">
+        <v>17</v>
+      </c>
+      <c r="B207" s="2">
+        <v>45908</v>
+      </c>
+      <c r="C207" s="3">
+        <v>0.43333333333333335</v>
+      </c>
+      <c r="D207">
+        <v>24.1</v>
+      </c>
+      <c r="E207">
+        <v>3</v>
+      </c>
+      <c r="I207">
+        <v>2.5</v>
+      </c>
+      <c r="J207">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="208" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A208" t="s">
+        <v>18</v>
+      </c>
+      <c r="B208" s="2">
+        <v>45908</v>
+      </c>
+      <c r="C208" s="3">
+        <v>0.4368055555555555</v>
+      </c>
+      <c r="D208">
+        <v>24.2</v>
+      </c>
+      <c r="E208">
+        <v>2</v>
+      </c>
+      <c r="F208">
+        <v>2.4</v>
+      </c>
+      <c r="G208">
+        <v>2.5</v>
+      </c>
+      <c r="H208">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="I208">
+        <v>2.5</v>
+      </c>
+      <c r="J208">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="209" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A209" t="s">
+        <v>19</v>
+      </c>
+      <c r="B209" s="2">
+        <v>45908</v>
+      </c>
+      <c r="C209" s="3">
+        <v>0.44027777777777777</v>
+      </c>
+      <c r="D209">
+        <v>23.4</v>
+      </c>
+      <c r="E209">
+        <v>1.8</v>
+      </c>
+      <c r="F209">
+        <v>1.8</v>
+      </c>
+      <c r="G209">
+        <v>1.9</v>
+      </c>
+      <c r="H209">
+        <v>1.7</v>
+      </c>
+      <c r="I209">
+        <v>2.5</v>
+      </c>
+      <c r="J209">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="210" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A210" t="s">
+        <v>20</v>
+      </c>
+      <c r="B210" s="2">
+        <v>45908</v>
+      </c>
+      <c r="C210" s="3">
+        <v>0.44375000000000003</v>
+      </c>
+      <c r="D210">
+        <v>23.6</v>
+      </c>
+      <c r="E210">
+        <v>1.9</v>
+      </c>
+      <c r="I210">
+        <v>2.5</v>
+      </c>
+      <c r="J210">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="211" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A211" t="s">
+        <v>21</v>
+      </c>
+      <c r="B211" s="2">
+        <v>45908</v>
+      </c>
+      <c r="C211" s="3">
+        <v>0.44722222222222219</v>
+      </c>
+      <c r="D211">
+        <v>23.6</v>
+      </c>
+      <c r="E211">
+        <v>2.4</v>
+      </c>
+      <c r="F211">
+        <v>2.4</v>
+      </c>
+      <c r="G211">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="H211">
+        <v>2.4</v>
+      </c>
+      <c r="I211">
+        <v>2.5</v>
+      </c>
+      <c r="J211">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="212" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A212" t="s">
+        <v>7</v>
+      </c>
+      <c r="B212" s="2">
+        <v>45912</v>
+      </c>
+      <c r="C212" s="3">
+        <v>0.40416666666666662</v>
+      </c>
+      <c r="D212">
+        <v>24.5</v>
+      </c>
+      <c r="E212">
+        <v>5</v>
+      </c>
+      <c r="F212">
+        <v>4.5</v>
+      </c>
+      <c r="G212">
+        <v>4.8</v>
+      </c>
+      <c r="H212">
+        <v>5.4</v>
+      </c>
+      <c r="I212">
+        <v>2.5</v>
+      </c>
+      <c r="J212">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="213" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A213" t="s">
+        <v>8</v>
+      </c>
+      <c r="B213" s="2">
+        <v>45912</v>
+      </c>
+      <c r="C213" s="3">
+        <v>0.40763888888888888</v>
+      </c>
+      <c r="D213">
+        <v>23.7</v>
+      </c>
+      <c r="E213">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="F213">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="G213">
+        <v>5.2</v>
+      </c>
+      <c r="H213">
+        <v>5.5</v>
+      </c>
+      <c r="I213">
+        <v>2.5</v>
+      </c>
+      <c r="J213">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="214" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A214" t="s">
+        <v>9</v>
+      </c>
+      <c r="B214" s="2">
+        <v>45912</v>
+      </c>
+      <c r="C214" s="3">
+        <v>0.41111111111111115</v>
+      </c>
+      <c r="D214">
+        <v>24.7</v>
+      </c>
+      <c r="E214">
+        <v>4.8</v>
+      </c>
+      <c r="F214">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="G214">
+        <v>5.5</v>
+      </c>
+      <c r="H214">
+        <v>5.2</v>
+      </c>
+      <c r="I214">
+        <v>2.5</v>
+      </c>
+      <c r="J214">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="215" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A215" t="s">
+        <v>10</v>
+      </c>
+      <c r="B215" s="2">
+        <v>45912</v>
+      </c>
+      <c r="C215" s="3">
+        <v>0.4145833333333333</v>
+      </c>
+      <c r="D215">
+        <v>24.9</v>
+      </c>
+      <c r="E215">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="F215">
+        <v>5</v>
+      </c>
+      <c r="G215">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="H215">
+        <v>4.8</v>
+      </c>
+      <c r="I215">
+        <v>2.5</v>
+      </c>
+      <c r="J215">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="216" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A216" t="s">
+        <v>11</v>
+      </c>
+      <c r="B216" s="2">
+        <v>45912</v>
+      </c>
+      <c r="C216" s="3">
+        <v>0.41736111111111113</v>
+      </c>
+      <c r="D216">
+        <v>24.2</v>
+      </c>
+      <c r="E216">
+        <v>3.5</v>
+      </c>
+      <c r="F216">
+        <v>3.5</v>
+      </c>
+      <c r="G216">
+        <v>4</v>
+      </c>
+      <c r="H216">
+        <v>3.8</v>
+      </c>
+      <c r="I216">
+        <v>2.5</v>
+      </c>
+      <c r="J216">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="217" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A217" t="s">
+        <v>12</v>
+      </c>
+      <c r="B217" s="2">
+        <v>45912</v>
+      </c>
+      <c r="C217" s="3">
+        <v>0.42222222222222222</v>
+      </c>
+      <c r="D217">
+        <v>25.7</v>
+      </c>
+      <c r="E217">
+        <v>5</v>
+      </c>
+      <c r="F217">
+        <v>4.7</v>
+      </c>
+      <c r="G217">
+        <v>5.9</v>
+      </c>
+      <c r="H217">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="I217">
+        <v>2.5</v>
+      </c>
+      <c r="J217">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="218" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A218" t="s">
+        <v>13</v>
+      </c>
+      <c r="B218" s="2">
+        <v>45912</v>
+      </c>
+      <c r="C218" s="3">
+        <v>0.42569444444444443</v>
+      </c>
+      <c r="D218">
+        <v>24.8</v>
+      </c>
+      <c r="E218">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="F218">
+        <v>5</v>
+      </c>
+      <c r="G218">
+        <v>5.4</v>
+      </c>
+      <c r="H218">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="I218">
+        <v>2.5</v>
+      </c>
+      <c r="J218">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="219" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A219" t="s">
+        <v>14</v>
+      </c>
+      <c r="B219" s="2">
+        <v>45912</v>
+      </c>
+      <c r="C219" s="3">
+        <v>0.4291666666666667</v>
+      </c>
+      <c r="D219">
+        <v>25.1</v>
+      </c>
+      <c r="E219">
+        <v>5.5</v>
+      </c>
+      <c r="I219">
+        <v>2.5</v>
+      </c>
+      <c r="J219">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="220" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A220" t="s">
+        <v>15</v>
+      </c>
+      <c r="B220" s="2">
+        <v>45912</v>
+      </c>
+      <c r="C220" s="3">
+        <v>0.43263888888888885</v>
+      </c>
+      <c r="D220">
+        <v>25.9</v>
+      </c>
+      <c r="E220">
+        <v>4.8</v>
+      </c>
+      <c r="F220">
+        <v>5.2</v>
+      </c>
+      <c r="G220">
+        <v>5</v>
+      </c>
+      <c r="H220">
+        <v>5.3</v>
+      </c>
+      <c r="I220">
+        <v>2.5</v>
+      </c>
+      <c r="J220">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="221" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A221" t="s">
+        <v>16</v>
+      </c>
+      <c r="B221" s="2">
+        <v>45912</v>
+      </c>
+      <c r="C221" s="3">
+        <v>0.43611111111111112</v>
+      </c>
+      <c r="D221">
+        <v>25.6</v>
+      </c>
+      <c r="E221">
+        <v>5.9</v>
+      </c>
+      <c r="I221">
+        <v>2.5</v>
+      </c>
+      <c r="J221">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="222" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A222" t="s">
+        <v>17</v>
+      </c>
+      <c r="B222" s="2">
+        <v>45912</v>
+      </c>
+      <c r="C222" s="3">
+        <v>0.4458333333333333</v>
+      </c>
+      <c r="D222">
+        <v>27</v>
+      </c>
+      <c r="E222">
+        <v>4.5</v>
+      </c>
+      <c r="F222">
+        <v>5.9</v>
+      </c>
+      <c r="G222">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="H222">
+        <v>4.2</v>
+      </c>
+      <c r="I222">
+        <v>2.5</v>
+      </c>
+      <c r="J222">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="223" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A223" t="s">
+        <v>18</v>
+      </c>
+      <c r="B223" s="2">
+        <v>45912</v>
+      </c>
+      <c r="C223" s="3">
+        <v>0.45</v>
+      </c>
+      <c r="D223">
+        <v>26.2</v>
+      </c>
+      <c r="E223">
+        <v>5</v>
+      </c>
+      <c r="F223">
+        <v>5.3</v>
+      </c>
+      <c r="G223">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="H223">
+        <v>5</v>
+      </c>
+      <c r="I223">
+        <v>2.5</v>
+      </c>
+      <c r="J223">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="224" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A224" t="s">
+        <v>19</v>
+      </c>
+      <c r="B224" s="2">
+        <v>45912</v>
+      </c>
+      <c r="C224" s="3">
+        <v>0.45347222222222222</v>
+      </c>
+      <c r="D224">
+        <v>25.9</v>
+      </c>
+      <c r="E224">
+        <v>5</v>
+      </c>
+      <c r="I224">
+        <v>2.5</v>
+      </c>
+      <c r="J224">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="225" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A225" t="s">
+        <v>20</v>
+      </c>
+      <c r="B225" s="2">
+        <v>45912</v>
+      </c>
+      <c r="C225" s="3">
+        <v>0.45694444444444443</v>
+      </c>
+      <c r="D225">
+        <v>26.7</v>
+      </c>
+      <c r="E225">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="F225">
+        <v>4.7</v>
+      </c>
+      <c r="G225">
+        <v>4.8</v>
+      </c>
+      <c r="H225">
+        <v>4.7</v>
+      </c>
+      <c r="I225">
+        <v>2.5</v>
+      </c>
+      <c r="J225">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="226" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A226" t="s">
+        <v>21</v>
+      </c>
+      <c r="B226" s="2">
+        <v>45912</v>
+      </c>
+      <c r="C226" s="3">
+        <v>0.4604166666666667</v>
+      </c>
+      <c r="D226">
+        <v>28</v>
+      </c>
+      <c r="E226">
+        <v>5.6</v>
+      </c>
+      <c r="I226">
+        <v>2.5</v>
+      </c>
+      <c r="J226">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="227" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A227" t="s">
+        <v>7</v>
+      </c>
+      <c r="B227" s="2">
+        <v>45918</v>
+      </c>
+      <c r="C227" s="3">
+        <v>0.51944444444444449</v>
+      </c>
+      <c r="D227">
+        <v>30.8</v>
+      </c>
+      <c r="E227">
+        <v>5</v>
+      </c>
+      <c r="F227">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="G227">
+        <v>5</v>
+      </c>
+      <c r="H227">
+        <v>6</v>
+      </c>
+      <c r="I227">
+        <v>2.5</v>
+      </c>
+      <c r="J227">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="228" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A228" t="s">
+        <v>8</v>
+      </c>
+      <c r="B228" s="2">
+        <v>45918</v>
+      </c>
+      <c r="C228" s="3">
+        <v>0.5229166666666667</v>
+      </c>
+      <c r="D228">
+        <v>33.1</v>
+      </c>
+      <c r="E228">
+        <v>6</v>
+      </c>
+      <c r="F228">
+        <v>5.5</v>
+      </c>
+      <c r="G228">
+        <v>5.9</v>
+      </c>
+      <c r="H228">
+        <v>7.2</v>
+      </c>
+      <c r="I228">
+        <v>2.5</v>
+      </c>
+      <c r="J228">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="229" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A229" t="s">
+        <v>9</v>
+      </c>
+      <c r="B229" s="2">
+        <v>45918</v>
+      </c>
+      <c r="C229" s="3">
+        <v>0.52638888888888891</v>
+      </c>
+      <c r="D229">
+        <v>32.299999999999997</v>
+      </c>
+      <c r="E229">
+        <v>5</v>
+      </c>
+      <c r="F229">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="G229">
+        <v>5</v>
+      </c>
+      <c r="H229">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="I229">
+        <v>2.5</v>
+      </c>
+      <c r="J229">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="230" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A230" t="s">
+        <v>10</v>
+      </c>
+      <c r="B230" s="2">
+        <v>45918</v>
+      </c>
+      <c r="C230" s="3">
+        <v>0.52986111111111112</v>
+      </c>
+      <c r="D230">
+        <v>33</v>
+      </c>
+      <c r="E230">
+        <v>5.3</v>
+      </c>
+      <c r="F230">
+        <v>5</v>
+      </c>
+      <c r="G230">
+        <v>4.5</v>
+      </c>
+      <c r="H230">
+        <v>5.8</v>
+      </c>
+      <c r="I230">
+        <v>2.5</v>
+      </c>
+      <c r="J230">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="231" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A231" t="s">
+        <v>11</v>
+      </c>
+      <c r="B231" s="2">
+        <v>45918</v>
+      </c>
+      <c r="C231" s="3">
+        <v>0.53333333333333333</v>
+      </c>
+      <c r="D231">
+        <v>30.7</v>
+      </c>
+      <c r="E231">
+        <v>6</v>
+      </c>
+      <c r="F231">
+        <v>5</v>
+      </c>
+      <c r="G231">
+        <v>6.2</v>
+      </c>
+      <c r="H231">
+        <v>7.9</v>
+      </c>
+      <c r="I231">
+        <v>2.5</v>
+      </c>
+      <c r="J231">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="232" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A232" t="s">
+        <v>12</v>
+      </c>
+      <c r="B232" s="2">
+        <v>45918</v>
+      </c>
+      <c r="C232" s="3">
+        <v>0.53680555555555554</v>
+      </c>
+      <c r="D232">
+        <v>30.2</v>
+      </c>
+      <c r="E232">
+        <v>7.2</v>
+      </c>
+      <c r="F232">
+        <v>4</v>
+      </c>
+      <c r="G232">
+        <v>5.4</v>
+      </c>
+      <c r="H232">
+        <v>7</v>
+      </c>
+      <c r="I232">
+        <v>2.5</v>
+      </c>
+      <c r="J232">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="233" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A233" t="s">
+        <v>13</v>
+      </c>
+      <c r="B233" s="2">
+        <v>45918</v>
+      </c>
+      <c r="C233" s="3">
+        <v>0.54027777777777775</v>
+      </c>
+      <c r="D233">
+        <v>29.4</v>
+      </c>
+      <c r="E233">
+        <v>5.6</v>
+      </c>
+      <c r="F233">
+        <v>5.9</v>
+      </c>
+      <c r="G233">
+        <v>4.5</v>
+      </c>
+      <c r="H233">
+        <v>6</v>
+      </c>
+      <c r="I233">
+        <v>2.5</v>
+      </c>
+      <c r="J233">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="234" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A234" t="s">
+        <v>14</v>
+      </c>
+      <c r="B234" s="2">
+        <v>45918</v>
+      </c>
+      <c r="C234" s="3">
+        <v>0.54375000000000007</v>
+      </c>
+      <c r="D234">
+        <v>30.1</v>
+      </c>
+      <c r="E234">
+        <v>6.6</v>
+      </c>
+      <c r="F234">
+        <v>5</v>
+      </c>
+      <c r="G234">
+        <v>5.9</v>
+      </c>
+      <c r="H234">
+        <v>5.4</v>
+      </c>
+      <c r="I234">
+        <v>2.5</v>
+      </c>
+      <c r="J234">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="235" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A235" t="s">
+        <v>15</v>
+      </c>
+      <c r="B235" s="2">
+        <v>45918</v>
+      </c>
+      <c r="C235" s="3">
+        <v>0.54722222222222217</v>
+      </c>
+      <c r="D235">
+        <v>30.7</v>
+      </c>
+      <c r="E235">
+        <v>7.5</v>
+      </c>
+      <c r="F235">
+        <v>6.5</v>
+      </c>
+      <c r="G235">
+        <v>7.9</v>
+      </c>
+      <c r="H235">
+        <v>7.1</v>
+      </c>
+      <c r="I235">
+        <v>2.5</v>
+      </c>
+      <c r="J235">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="236" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A236" t="s">
+        <v>16</v>
+      </c>
+      <c r="B236" s="2">
+        <v>45918</v>
+      </c>
+      <c r="C236" s="3">
+        <v>0.55069444444444449</v>
+      </c>
+      <c r="D236">
+        <v>29.9</v>
+      </c>
+      <c r="E236">
+        <v>9.1</v>
+      </c>
+      <c r="F236">
+        <v>6.1</v>
+      </c>
+      <c r="G236">
+        <v>6.2</v>
+      </c>
+      <c r="H236">
+        <v>6.6</v>
+      </c>
+      <c r="I236">
+        <v>2.5</v>
+      </c>
+      <c r="J236">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="237" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A237" t="s">
+        <v>17</v>
+      </c>
+      <c r="B237" s="2">
+        <v>45918</v>
+      </c>
+      <c r="C237" s="3">
+        <v>0.5541666666666667</v>
+      </c>
+      <c r="D237">
+        <v>29.8</v>
+      </c>
+      <c r="E237">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="F237">
+        <v>5.5</v>
+      </c>
+      <c r="G237">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="H237">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="I237">
+        <v>2.5</v>
+      </c>
+      <c r="J237">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="238" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A238" t="s">
+        <v>18</v>
+      </c>
+      <c r="B238" s="2">
+        <v>45918</v>
+      </c>
+      <c r="C238" s="3">
+        <v>0.55763888888888891</v>
+      </c>
+      <c r="D238">
+        <v>29.4</v>
+      </c>
+      <c r="E238">
+        <v>6.5</v>
+      </c>
+      <c r="F238">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="G238">
+        <v>3.1</v>
+      </c>
+      <c r="H238">
+        <v>4.5</v>
+      </c>
+      <c r="I238">
+        <v>2.5</v>
+      </c>
+      <c r="J238">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="239" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A239" t="s">
+        <v>19</v>
+      </c>
+      <c r="B239" s="2">
+        <v>45918</v>
+      </c>
+      <c r="C239" s="3">
+        <v>0.56111111111111101</v>
+      </c>
+      <c r="D239">
+        <v>30.4</v>
+      </c>
+      <c r="E239">
+        <v>6.6</v>
+      </c>
+      <c r="F239">
+        <v>5.6</v>
+      </c>
+      <c r="G239">
+        <v>5.9</v>
+      </c>
+      <c r="H239">
+        <v>7</v>
+      </c>
+      <c r="I239">
+        <v>2.5</v>
+      </c>
+      <c r="J239">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="240" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A240" t="s">
+        <v>20</v>
+      </c>
+      <c r="B240" s="2">
+        <v>45918</v>
+      </c>
+      <c r="C240" s="3">
+        <v>0.56458333333333299</v>
+      </c>
+      <c r="D240">
+        <v>31</v>
+      </c>
+      <c r="E240">
+        <v>7.1</v>
+      </c>
+      <c r="F240">
+        <v>6.6</v>
+      </c>
+      <c r="G240">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="H240">
+        <v>7.5</v>
+      </c>
+      <c r="I240">
+        <v>2.5</v>
+      </c>
+      <c r="J240">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="241" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A241" t="s">
+        <v>21</v>
+      </c>
+      <c r="B241" s="2">
+        <v>45918</v>
+      </c>
+      <c r="C241" s="3">
+        <v>0.56874999999999998</v>
+      </c>
+      <c r="D241">
+        <v>30.5</v>
+      </c>
+      <c r="E241">
+        <v>7.5</v>
+      </c>
+      <c r="F241">
+        <v>7</v>
+      </c>
+      <c r="G241">
+        <v>6.9</v>
+      </c>
+      <c r="H241">
+        <v>8</v>
+      </c>
+      <c r="I241">
+        <v>2.5</v>
+      </c>
+      <c r="J241">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="242" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A242" t="s">
+        <v>7</v>
+      </c>
+      <c r="B242" s="2">
+        <v>45924</v>
+      </c>
+    </row>
+    <row r="243" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A243" t="s">
+        <v>8</v>
+      </c>
+      <c r="B243" s="2">
+        <v>45924</v>
+      </c>
+    </row>
+    <row r="244" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A244" t="s">
+        <v>9</v>
+      </c>
+      <c r="B244" s="2">
+        <v>45924</v>
+      </c>
+    </row>
+    <row r="245" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A245" t="s">
+        <v>10</v>
+      </c>
+      <c r="B245" s="2">
+        <v>45924</v>
+      </c>
+    </row>
+    <row r="246" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A246" t="s">
+        <v>11</v>
+      </c>
+      <c r="B246" s="2">
+        <v>45924</v>
+      </c>
+    </row>
+    <row r="247" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A247" t="s">
+        <v>12</v>
+      </c>
+      <c r="B247" s="2">
+        <v>45924</v>
+      </c>
+    </row>
+    <row r="248" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A248" t="s">
+        <v>13</v>
+      </c>
+      <c r="B248" s="2">
+        <v>45924</v>
+      </c>
+    </row>
+    <row r="249" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A249" t="s">
+        <v>14</v>
+      </c>
+      <c r="B249" s="2">
+        <v>45924</v>
+      </c>
+    </row>
+    <row r="250" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A250" t="s">
+        <v>15</v>
+      </c>
+      <c r="B250" s="2">
+        <v>45924</v>
+      </c>
+    </row>
+    <row r="251" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A251" t="s">
+        <v>16</v>
+      </c>
+      <c r="B251" s="2">
+        <v>45924</v>
+      </c>
+    </row>
+    <row r="252" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A252" t="s">
+        <v>17</v>
+      </c>
+      <c r="B252" s="2">
+        <v>45924</v>
+      </c>
+    </row>
+    <row r="253" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A253" t="s">
+        <v>18</v>
+      </c>
+      <c r="B253" s="2">
+        <v>45924</v>
+      </c>
+    </row>
+    <row r="254" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A254" t="s">
+        <v>19</v>
+      </c>
+      <c r="B254" s="2">
+        <v>45924</v>
+      </c>
+    </row>
+    <row r="255" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A255" t="s">
+        <v>20</v>
+      </c>
+      <c r="B255" s="2">
+        <v>45924</v>
+      </c>
+    </row>
+    <row r="256" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A256" t="s">
+        <v>21</v>
+      </c>
+      <c r="B256" s="2">
+        <v>45924</v>
       </c>
     </row>
   </sheetData>

</xml_diff>